<commit_message>
Đồng bộ dữ liệu khảo sát 2026-05-20
</commit_message>
<xml_diff>
--- a/data/khaosat.xlsx
+++ b/data/khaosat.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S358"/>
+  <dimension ref="A1:S372"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,7 +463,7 @@
         <v>5436</v>
       </c>
       <c r="B2" t="str">
-        <v>CS Bình Dương 2283</v>
+        <v>Cây trường 18 - T1</v>
       </c>
       <c r="C2" t="str">
         <v>11,3438654</v>
@@ -522,7 +522,7 @@
         <v>4870</v>
       </c>
       <c r="B3" t="str">
-        <v>Bình Dương 1756</v>
+        <v>Cây trường 19 - T1</v>
       </c>
       <c r="C3" t="str">
         <v>11,3434845</v>
@@ -581,7 +581,7 @@
         <v>5437</v>
       </c>
       <c r="B4" t="str">
-        <v>CS Bình Dương 2284</v>
+        <v>Cây trường 15 - T1</v>
       </c>
       <c r="C4" t="str">
         <v>11,3461486</v>
@@ -640,7 +640,7 @@
         <v>5432</v>
       </c>
       <c r="B5" t="str">
-        <v>CS Bình Dương 2279</v>
+        <v>Cây trường 16 - T1</v>
       </c>
       <c r="C5" t="str">
         <v>11,3410005</v>
@@ -699,7 +699,7 @@
         <v>4869</v>
       </c>
       <c r="B6" t="str">
-        <v>Bình Dương 1755</v>
+        <v>Cây trường 22 - T1</v>
       </c>
       <c r="C6" t="str">
         <v>11,3435008</v>
@@ -758,7 +758,7 @@
         <v>5433</v>
       </c>
       <c r="B7" t="str">
-        <v>CS Bình Dương 2280</v>
+        <v>Cây trường 13 - T1</v>
       </c>
       <c r="C7" t="str">
         <v>11,3414781</v>
@@ -817,7 +817,7 @@
         <v>4868</v>
       </c>
       <c r="B8" t="str">
-        <v>Bình Dương 1754</v>
+        <v>Cây trường 21 - T1</v>
       </c>
       <c r="C8" t="str">
         <v>11,3406307</v>
@@ -876,7 +876,7 @@
         <v>4867</v>
       </c>
       <c r="B9" t="str">
-        <v>Bình Dương 1753</v>
+        <v>Cây trường 23 - T1</v>
       </c>
       <c r="C9" t="str">
         <v>11,3430694</v>
@@ -935,7 +935,7 @@
         <v>5434</v>
       </c>
       <c r="B10" t="str">
-        <v>CS Bình Dương 2281</v>
+        <v>Cây trường 10 - T1</v>
       </c>
       <c r="C10" t="str">
         <v>11,3448126</v>
@@ -994,7 +994,7 @@
         <v>5429</v>
       </c>
       <c r="B11" t="str">
-        <v>CS Bình Dương 2276</v>
+        <v>Cây trường 09 - T1</v>
       </c>
       <c r="C11" t="str">
         <v>11,3416985</v>
@@ -1053,7 +1053,7 @@
         <v>4866</v>
       </c>
       <c r="B12" t="str">
-        <v>Bình Dương 1752</v>
+        <v>Cây trường 26 - T1</v>
       </c>
       <c r="C12" t="str">
         <v>11,3427639</v>
@@ -1112,7 +1112,7 @@
         <v>4865</v>
       </c>
       <c r="B13" t="str">
-        <v>Bình Dương 1751</v>
+        <v>Cây trường 25 - T1</v>
       </c>
       <c r="C13" t="str">
         <v>11,3412964</v>
@@ -1171,7 +1171,7 @@
         <v>5430</v>
       </c>
       <c r="B14" t="str">
-        <v>CS Bình Dương 2277</v>
+        <v>Cây trường 07 - T1</v>
       </c>
       <c r="C14" t="str">
         <v>11,3444389</v>
@@ -1230,7 +1230,7 @@
         <v>4864</v>
       </c>
       <c r="B15" t="str">
-        <v>Bình Dương 1750</v>
+        <v>Cây trường 28 - T1-</v>
       </c>
       <c r="C15" t="str">
         <v>11,3424616</v>
@@ -1289,7 +1289,7 @@
         <v>4863</v>
       </c>
       <c r="B16" t="str">
-        <v>Bình Dương 1749</v>
+        <v>Cây trường 27 - T1</v>
       </c>
       <c r="C16" t="str">
         <v>11,3425892</v>
@@ -1348,7 +1348,7 @@
         <v>5431</v>
       </c>
       <c r="B17" t="str">
-        <v>CS Bình Dương 2278</v>
+        <v>Cây trường 06 - T1</v>
       </c>
       <c r="C17" t="str">
         <v>11,3869819</v>
@@ -1407,7 +1407,7 @@
         <v>5426</v>
       </c>
       <c r="B18" t="str">
-        <v>CS Bình Dương 2273</v>
+        <v>TVT71-T5</v>
       </c>
       <c r="C18" t="str">
         <v>11,3859231</v>
@@ -1466,7 +1466,7 @@
         <v>5427</v>
       </c>
       <c r="B19" t="str">
-        <v>CS Bình Dương 2274</v>
+        <v>TVT71-T4</v>
       </c>
       <c r="C19" t="str">
         <v>11,3832698</v>
@@ -1525,7 +1525,7 @@
         <v>5428</v>
       </c>
       <c r="B20" t="str">
-        <v>CS Bình Dương 2275</v>
+        <v>TVT71-T3</v>
       </c>
       <c r="C20" t="str">
         <v>11,3807766</v>
@@ -1584,7 +1584,7 @@
         <v>4862</v>
       </c>
       <c r="B21" t="str">
-        <v>Bình Dương 1748</v>
+        <v>Cây trường 41-T1</v>
       </c>
       <c r="C21" t="str">
         <v>11,3355921</v>
@@ -1643,7 +1643,7 @@
         <v>5423</v>
       </c>
       <c r="B22" t="str">
-        <v>CS Bình Dương 2270</v>
+        <v>TVT71-T2</v>
       </c>
       <c r="C22" t="str">
         <v>11,3764306</v>
@@ -1702,7 +1702,7 @@
         <v>4861</v>
       </c>
       <c r="B23" t="str">
-        <v>Bình Dương 1747</v>
+        <v>Cây trường 40-T1</v>
       </c>
       <c r="C23" t="str">
         <v>11,3382415</v>
@@ -1761,7 +1761,7 @@
         <v>5424</v>
       </c>
       <c r="B24" t="str">
-        <v>CS Bình Dương 2271</v>
+        <v>TVT71-T1</v>
       </c>
       <c r="C24" t="str">
         <v>11,3650082</v>
@@ -1820,7 +1820,7 @@
         <v>4860</v>
       </c>
       <c r="B25" t="str">
-        <v>Bình Dương 1746</v>
+        <v>Cây trường 39-T1</v>
       </c>
       <c r="C25" t="str">
         <v>11,3325840</v>
@@ -1879,7 +1879,7 @@
         <v>4859</v>
       </c>
       <c r="B26" t="str">
-        <v>Bình Dương 1745</v>
+        <v>Cây trường 38-T1</v>
       </c>
       <c r="C26" t="str">
         <v>11,3361605</v>
@@ -1938,7 +1938,7 @@
         <v>4858</v>
       </c>
       <c r="B27" t="str">
-        <v>Bình Dương 1744</v>
+        <v>Cây trường 37-T1</v>
       </c>
       <c r="C27" t="str">
         <v>11,3382603</v>
@@ -1997,7 +1997,7 @@
         <v>5425</v>
       </c>
       <c r="B28" t="str">
-        <v>CS Bình Dương 2272</v>
+        <v>Cây trường 33-T1</v>
       </c>
       <c r="C28" t="str">
         <v>11,3461921</v>
@@ -2056,7 +2056,7 @@
         <v>4857</v>
       </c>
       <c r="B29" t="str">
-        <v>Bình Dương 1743</v>
+        <v>Cây trường 30-T1</v>
       </c>
       <c r="C29" t="str">
         <v>11,3430801</v>
@@ -2115,7 +2115,7 @@
         <v>4856</v>
       </c>
       <c r="B30" t="str">
-        <v>Bình Dương 1742</v>
+        <v>Cây trường 31-T1</v>
       </c>
       <c r="C30" t="str">
         <v>11,3422405</v>
@@ -2174,7 +2174,7 @@
         <v>4855</v>
       </c>
       <c r="B31" t="str">
-        <v>Bình Dương 1741</v>
+        <v>Cây trường 68-T1</v>
       </c>
       <c r="C31" t="str">
         <v>11,3185248</v>
@@ -2351,7 +2351,7 @@
         <v>5422</v>
       </c>
       <c r="B34" t="str">
-        <v>CS Bình Dương 2269</v>
+        <v>Lai Uyên 9 -T1</v>
       </c>
       <c r="C34" t="str">
         <v>11,3431082</v>
@@ -2410,7 +2410,7 @@
         <v>5419</v>
       </c>
       <c r="B35" t="str">
-        <v>CS Bình Dương 2266</v>
+        <v>Lai Uyên 10 -T1</v>
       </c>
       <c r="C35" t="str">
         <v>11,3422614</v>
@@ -2469,7 +2469,7 @@
         <v>5418</v>
       </c>
       <c r="B36" t="str">
-        <v>CS Bình Dương 2265</v>
+        <v>Lai Uyên 11-T1</v>
       </c>
       <c r="C36" t="str">
         <v>11,3384645</v>
@@ -2528,7 +2528,7 @@
         <v>5417</v>
       </c>
       <c r="B37" t="str">
-        <v>CS Bình Dương 2264</v>
+        <v>Lai Uyên 12-T1</v>
       </c>
       <c r="C37" t="str">
         <v>11,3382468</v>
@@ -2587,7 +2587,7 @@
         <v>4810</v>
       </c>
       <c r="B38" t="str">
-        <v>Bình Dương 1696</v>
+        <v>Lai Uyên 15-T1</v>
       </c>
       <c r="C38" t="str">
         <v>11,3327582</v>
@@ -2646,7 +2646,7 @@
         <v>4811</v>
       </c>
       <c r="B39" t="str">
-        <v>Bình Dương 1697</v>
+        <v>Lai Uyên 17-T1</v>
       </c>
       <c r="C39" t="str">
         <v>11,3297137</v>
@@ -2705,7 +2705,7 @@
         <v>4812</v>
       </c>
       <c r="B40" t="str">
-        <v>Bình Dương 1698</v>
+        <v>Lai Uyên 16-T1</v>
       </c>
       <c r="C40" t="str">
         <v>11,3300271</v>
@@ -2764,7 +2764,7 @@
         <v>4813</v>
       </c>
       <c r="B41" t="str">
-        <v>Bình Dương 1699</v>
+        <v>Lai Uyên 7-T1</v>
       </c>
       <c r="C41" t="str">
         <v>11,3320960</v>
@@ -2823,7 +2823,7 @@
         <v>4854</v>
       </c>
       <c r="B42" t="str">
-        <v>Bình Dương 1740</v>
+        <v>Cây trường 05 - T2</v>
       </c>
       <c r="C42" t="str">
         <v>11,3397621</v>
@@ -2882,7 +2882,7 @@
         <v>4814</v>
       </c>
       <c r="B43" t="str">
-        <v>Bình Dương 1700</v>
+        <v>Lai Uyên 6-T1</v>
       </c>
       <c r="C43" t="str">
         <v>11,3321023</v>
@@ -2941,7 +2941,7 @@
         <v>4853</v>
       </c>
       <c r="B44" t="str">
-        <v>Bình Dương 1739</v>
+        <v>Cây trường 05 - T1</v>
       </c>
       <c r="C44" t="str">
         <v>11,3413566</v>
@@ -3000,7 +3000,7 @@
         <v>4815</v>
       </c>
       <c r="B45" t="str">
-        <v>Bình Dương 1701</v>
+        <v>Lai Uyên 4-T1</v>
       </c>
       <c r="C45" t="str">
         <v>11,3365433</v>
@@ -3059,7 +3059,7 @@
         <v>4852</v>
       </c>
       <c r="B46" t="str">
-        <v>Bình Dương 1738</v>
+        <v>Cây trường 03 - T1</v>
       </c>
       <c r="C46" t="str">
         <v>11,3432353</v>
@@ -3118,7 +3118,7 @@
         <v>4816</v>
       </c>
       <c r="B47" t="str">
-        <v>Bình Dương 1702</v>
+        <v>Lai Uyên 3-T1</v>
       </c>
       <c r="C47" t="str">
         <v>11,3401893</v>
@@ -3177,7 +3177,7 @@
         <v>4817</v>
       </c>
       <c r="B48" t="str">
-        <v>Bình Dương 1703</v>
+        <v>Lai Uyên 2 -T1</v>
       </c>
       <c r="C48" t="str">
         <v>11,3420700</v>
@@ -3236,7 +3236,7 @@
         <v>4818</v>
       </c>
       <c r="B49" t="str">
-        <v>Bình Dương 1704</v>
+        <v>TVT25-T2</v>
       </c>
       <c r="C49" t="str">
         <v>11,3458199</v>
@@ -3295,7 +3295,7 @@
         <v>4819</v>
       </c>
       <c r="B50" t="str">
-        <v>Bình Dương 1705</v>
+        <v>TVT25-T1</v>
       </c>
       <c r="C50" t="str">
         <v>11,3531247</v>
@@ -3354,7 +3354,7 @@
         <v>4851</v>
       </c>
       <c r="B51" t="str">
-        <v>Bình Dương 1737</v>
+        <v>TVT - đường 08 - T1</v>
       </c>
       <c r="C51" t="str">
         <v>11,3569689</v>
@@ -3413,7 +3413,7 @@
         <v>4821</v>
       </c>
       <c r="B52" t="str">
-        <v>Bình Dương 1707</v>
+        <v>TVT131-T3</v>
       </c>
       <c r="C52" t="str">
         <v>11,3618684</v>
@@ -3472,7 +3472,7 @@
         <v>4850</v>
       </c>
       <c r="B53" t="str">
-        <v>Bình Dương 1736</v>
+        <v>TVT - đường 10 - T1</v>
       </c>
       <c r="C53" t="str">
         <v>11,3528641</v>
@@ -3531,7 +3531,7 @@
         <v>4824</v>
       </c>
       <c r="B54" t="str">
-        <v>Bình Dương 1710</v>
+        <v>TVT131-T2</v>
       </c>
       <c r="C54" t="str">
         <v>11,3620872</v>
@@ -3590,7 +3590,7 @@
         <v>4823</v>
       </c>
       <c r="B55" t="str">
-        <v>Bình Dương 1709</v>
+        <v>TVT131-T1</v>
       </c>
       <c r="C55" t="str">
         <v>11,3644495</v>
@@ -3649,7 +3649,7 @@
         <v>4822</v>
       </c>
       <c r="B56" t="str">
-        <v>Bình Dương 1708</v>
+        <v>TVT124-T1</v>
       </c>
       <c r="C56" t="str">
         <v>11,3663921</v>
@@ -3708,7 +3708,7 @@
         <v>4827</v>
       </c>
       <c r="B57" t="str">
-        <v>Bình Dương 1713</v>
+        <v>TVT 04-T1</v>
       </c>
       <c r="C57" t="str">
         <v>11,3479744</v>
@@ -3767,7 +3767,7 @@
         <v>4849</v>
       </c>
       <c r="B58" t="str">
-        <v>Bình Dương 1735</v>
+        <v>TVT - đường 18 - T1</v>
       </c>
       <c r="C58" t="str">
         <v>11,3471247</v>
@@ -3826,7 +3826,7 @@
         <v>4826</v>
       </c>
       <c r="B59" t="str">
-        <v>Bình Dương 1712</v>
+        <v>Cây trường 02-T1</v>
       </c>
       <c r="C59" t="str">
         <v>11,3460680</v>
@@ -3885,7 +3885,7 @@
         <v>5575</v>
       </c>
       <c r="B60" t="str">
-        <v>ĐT750</v>
+        <v>ĐT750 - T5</v>
       </c>
       <c r="C60" t="str">
         <v>11,3442438</v>
@@ -3944,7 +3944,7 @@
         <v>4825</v>
       </c>
       <c r="B61" t="str">
-        <v>Bình Dương 1711</v>
+        <v>Cây trường 51-T1</v>
       </c>
       <c r="C61" t="str">
         <v>11,2995189</v>
@@ -4003,7 +4003,7 @@
         <v>4848</v>
       </c>
       <c r="B62" t="str">
-        <v>Bình Dương 1734</v>
+        <v>ĐT750 - T4</v>
       </c>
       <c r="C62" t="str">
         <v>11,3447745</v>
@@ -4062,7 +4062,7 @@
         <v>4830</v>
       </c>
       <c r="B63" t="str">
-        <v>Bình Dương 1716</v>
+        <v>Cây trường 48-T1</v>
       </c>
       <c r="C63" t="str">
         <v>11,3156877</v>
@@ -4121,7 +4121,7 @@
         <v>4847</v>
       </c>
       <c r="B64" t="str">
-        <v>Bình Dương 1733</v>
+        <v>ĐT750 - T3</v>
       </c>
       <c r="C64" t="str">
         <v>11,3422511</v>
@@ -4180,7 +4180,7 @@
         <v>4829</v>
       </c>
       <c r="B65" t="str">
-        <v>Bình Dương 1715</v>
+        <v>Cây trường 69-T1</v>
       </c>
       <c r="C65" t="str">
         <v>11,3148616</v>
@@ -4239,7 +4239,7 @@
         <v>4846</v>
       </c>
       <c r="B66" t="str">
-        <v>Bình Dương 1732</v>
+        <v>Cây trường 14 - T1</v>
       </c>
       <c r="C66" t="str">
         <v>11,3463159</v>
@@ -4298,7 +4298,7 @@
         <v>4828</v>
       </c>
       <c r="B67" t="str">
-        <v>Bình Dương 1714</v>
+        <v>Cây trường 47-T1</v>
       </c>
       <c r="C67" t="str">
         <v>11,3206417</v>
@@ -4357,7 +4357,7 @@
         <v>4844</v>
       </c>
       <c r="B68" t="str">
-        <v>Bình Dương 1730</v>
+        <v>ĐT750 - T2</v>
       </c>
       <c r="C68" t="str">
         <v>11,3443087</v>
@@ -4416,7 +4416,7 @@
         <v>4833</v>
       </c>
       <c r="B69" t="str">
-        <v>Bình Dương 1719</v>
+        <v>Cây trường 35-T1</v>
       </c>
       <c r="C69" t="str">
         <v>11,3393666</v>
@@ -4475,7 +4475,7 @@
         <v>4905</v>
       </c>
       <c r="B70" t="str">
-        <v>Bình Dương 1791</v>
+        <v>Cây trường 34-T1</v>
       </c>
       <c r="C70" t="str">
         <v>11,3402417</v>
@@ -17930,25 +17930,25 @@
         <v>Lai Uyên-55</v>
       </c>
       <c r="C298" t="str">
-        <v>11,3077160</v>
+        <v>11,3079009</v>
       </c>
       <c r="D298" t="str">
-        <v>106,6321799</v>
+        <v>106,6317900</v>
       </c>
       <c r="E298" t="str">
         <v>Bến Lớn, Xã Bàu Bàng, Thành phố Hồ Chí Minh, 75751, Việt Nam</v>
       </c>
       <c r="F298" t="str">
-        <v>NGUYỄN NGỌC THẾ</v>
+        <v>Phạm Văn Tính</v>
       </c>
       <c r="G298" t="str">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H298" t="str">
         <v>101.246.000</v>
       </c>
       <c r="I298" t="str">
-        <v/>
+        <v>Tủ chiếu sáng nổi</v>
       </c>
       <c r="J298" t="str">
         <v/>
@@ -17963,13 +17963,13 @@
         <v/>
       </c>
       <c r="N298" t="str">
-        <v/>
+        <v>11:02:49 18/5/2026</v>
       </c>
       <c r="O298" t="str">
-        <v/>
+        <v>Lai Uyên 73</v>
       </c>
       <c r="P298" t="str">
-        <v/>
+        <v>1810</v>
       </c>
       <c r="Q298" t="str">
         <v/>
@@ -17978,7 +17978,7 @@
         <v/>
       </c>
       <c r="S298" t="str">
-        <v>Xã Bàu Bàng</v>
+        <v>Bến Lớn</v>
       </c>
     </row>
     <row r="299">
@@ -21521,9 +21521,835 @@
         <v>Bến Lớn</v>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v/>
+      </c>
+      <c r="B359" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="C359" t="str">
+        <v>11,3080246</v>
+      </c>
+      <c r="D359" t="str">
+        <v>106,6309400</v>
+      </c>
+      <c r="E359" t="str">
+        <v/>
+      </c>
+      <c r="F359" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G359" t="str">
+        <v>3</v>
+      </c>
+      <c r="H359" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I359" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J359" t="str">
+        <v/>
+      </c>
+      <c r="K359" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L359" t="str">
+        <v>250</v>
+      </c>
+      <c r="M359" t="str">
+        <v/>
+      </c>
+      <c r="N359" t="str">
+        <v>08:40:52 18/5/2026</v>
+      </c>
+      <c r="O359" t="str">
+        <v/>
+      </c>
+      <c r="P359" t="str">
+        <v/>
+      </c>
+      <c r="Q359" t="str">
+        <v/>
+      </c>
+      <c r="R359" t="str">
+        <v>Lai Uyên 55</v>
+      </c>
+      <c r="S359" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v/>
+      </c>
+      <c r="B360" t="str">
+        <v>Lu55_LU55_1_2</v>
+      </c>
+      <c r="C360" t="str">
+        <v>11,3080063</v>
+      </c>
+      <c r="D360" t="str">
+        <v>106,6313665</v>
+      </c>
+      <c r="E360" t="str">
+        <v/>
+      </c>
+      <c r="F360" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G360" t="str">
+        <v>3</v>
+      </c>
+      <c r="H360" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I360" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J360" t="str">
+        <v/>
+      </c>
+      <c r="K360" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L360" t="str">
+        <v>250</v>
+      </c>
+      <c r="M360" t="str">
+        <v/>
+      </c>
+      <c r="N360" t="str">
+        <v>08:41:11 18/5/2026</v>
+      </c>
+      <c r="O360" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P360" t="str">
+        <v>17</v>
+      </c>
+      <c r="Q360" t="str">
+        <v/>
+      </c>
+      <c r="R360" t="str">
+        <v/>
+      </c>
+      <c r="S360" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v/>
+      </c>
+      <c r="B361" t="str">
+        <v>Lu55_LU55_1_3</v>
+      </c>
+      <c r="C361" t="str">
+        <v>11,3079170</v>
+      </c>
+      <c r="D361" t="str">
+        <v>106,6321832</v>
+      </c>
+      <c r="E361" t="str">
+        <v/>
+      </c>
+      <c r="F361" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G361" t="str">
+        <v>4</v>
+      </c>
+      <c r="H361" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I361" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J361" t="str">
+        <v/>
+      </c>
+      <c r="K361" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L361" t="str">
+        <v>250</v>
+      </c>
+      <c r="M361" t="str">
+        <v/>
+      </c>
+      <c r="N361" t="str">
+        <v>10:55:41 18/5/2026</v>
+      </c>
+      <c r="O361" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P361" t="str">
+        <v>138</v>
+      </c>
+      <c r="Q361" t="str">
+        <v/>
+      </c>
+      <c r="R361" t="str">
+        <v/>
+      </c>
+      <c r="S361" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v/>
+      </c>
+      <c r="B362" t="str">
+        <v>Lu55_LU55_1_4</v>
+      </c>
+      <c r="C362" t="str">
+        <v>11,3078374</v>
+      </c>
+      <c r="D362" t="str">
+        <v>106,6328250</v>
+      </c>
+      <c r="E362" t="str">
+        <v/>
+      </c>
+      <c r="F362" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G362" t="str">
+        <v>4</v>
+      </c>
+      <c r="H362" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I362" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J362" t="str">
+        <v/>
+      </c>
+      <c r="K362" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L362" t="str">
+        <v>250</v>
+      </c>
+      <c r="M362" t="str">
+        <v/>
+      </c>
+      <c r="N362" t="str">
+        <v>10:55:46 18/5/2026</v>
+      </c>
+      <c r="O362" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P362" t="str">
+        <v>207</v>
+      </c>
+      <c r="Q362" t="str">
+        <v/>
+      </c>
+      <c r="R362" t="str">
+        <v/>
+      </c>
+      <c r="S362" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v/>
+      </c>
+      <c r="B363" t="str">
+        <v>Lu55_LU55_1_5</v>
+      </c>
+      <c r="C363" t="str">
+        <v>11,3077435</v>
+      </c>
+      <c r="D363" t="str">
+        <v>106,6332418</v>
+      </c>
+      <c r="E363" t="str">
+        <v/>
+      </c>
+      <c r="F363" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G363" t="str">
+        <v>4</v>
+      </c>
+      <c r="H363" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I363" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J363" t="str">
+        <v/>
+      </c>
+      <c r="K363" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L363" t="str">
+        <v>250</v>
+      </c>
+      <c r="M363" t="str">
+        <v/>
+      </c>
+      <c r="N363" t="str">
+        <v>10:57:31 18/5/2026</v>
+      </c>
+      <c r="O363" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P363" t="str">
+        <v>182</v>
+      </c>
+      <c r="Q363" t="str">
+        <v/>
+      </c>
+      <c r="R363" t="str">
+        <v/>
+      </c>
+      <c r="S363" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v/>
+      </c>
+      <c r="B364" t="str">
+        <v>Lu55_LU55_1_6</v>
+      </c>
+      <c r="C364" t="str">
+        <v>11,3075723</v>
+      </c>
+      <c r="D364" t="str">
+        <v>106,6339195</v>
+      </c>
+      <c r="E364" t="str">
+        <v/>
+      </c>
+      <c r="F364" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G364" t="str">
+        <v>4</v>
+      </c>
+      <c r="H364" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I364" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J364" t="str">
+        <v/>
+      </c>
+      <c r="K364" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L364" t="str">
+        <v>250</v>
+      </c>
+      <c r="M364" t="str">
+        <v/>
+      </c>
+      <c r="N364" t="str">
+        <v>10:58:07 18/5/2026</v>
+      </c>
+      <c r="O364" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P364" t="str">
+        <v>288</v>
+      </c>
+      <c r="Q364" t="str">
+        <v/>
+      </c>
+      <c r="R364" t="str">
+        <v/>
+      </c>
+      <c r="S364" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v/>
+      </c>
+      <c r="B365" t="str">
+        <v>Lu55_LU55_1_7</v>
+      </c>
+      <c r="C365" t="str">
+        <v>11,3073821</v>
+      </c>
+      <c r="D365" t="str">
+        <v>106,6346030</v>
+      </c>
+      <c r="E365" t="str">
+        <v/>
+      </c>
+      <c r="F365" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G365" t="str">
+        <v>4</v>
+      </c>
+      <c r="H365" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I365" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J365" t="str">
+        <v/>
+      </c>
+      <c r="K365" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L365" t="str">
+        <v>250</v>
+      </c>
+      <c r="M365" t="str">
+        <v/>
+      </c>
+      <c r="N365" t="str">
+        <v>10:58:06 18/5/2026</v>
+      </c>
+      <c r="O365" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P365" t="str">
+        <v>373</v>
+      </c>
+      <c r="Q365" t="str">
+        <v/>
+      </c>
+      <c r="R365" t="str">
+        <v/>
+      </c>
+      <c r="S365" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v/>
+      </c>
+      <c r="B366" t="str">
+        <v>Lu55_LU55_1_8</v>
+      </c>
+      <c r="C366" t="str">
+        <v>11,3071876</v>
+      </c>
+      <c r="D366" t="str">
+        <v>106,6356286</v>
+      </c>
+      <c r="E366" t="str">
+        <v/>
+      </c>
+      <c r="F366" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G366" t="str">
+        <v>3</v>
+      </c>
+      <c r="H366" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I366" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J366" t="str">
+        <v/>
+      </c>
+      <c r="K366" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L366" t="str">
+        <v>250</v>
+      </c>
+      <c r="M366" t="str">
+        <v/>
+      </c>
+      <c r="N366" t="str">
+        <v>08:34:55 18/5/2026</v>
+      </c>
+      <c r="O366" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P366" t="str">
+        <v>519</v>
+      </c>
+      <c r="Q366" t="str">
+        <v/>
+      </c>
+      <c r="R366" t="str">
+        <v/>
+      </c>
+      <c r="S366" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v/>
+      </c>
+      <c r="B367" t="str">
+        <v>Lu55_LU55_1_9</v>
+      </c>
+      <c r="C367" t="str">
+        <v>11,3070300</v>
+      </c>
+      <c r="D367" t="str">
+        <v>106,6361292</v>
+      </c>
+      <c r="E367" t="str">
+        <v/>
+      </c>
+      <c r="F367" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G367" t="str">
+        <v>3</v>
+      </c>
+      <c r="H367" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I367" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J367" t="str">
+        <v/>
+      </c>
+      <c r="K367" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L367" t="str">
+        <v>250</v>
+      </c>
+      <c r="M367" t="str">
+        <v/>
+      </c>
+      <c r="N367" t="str">
+        <v>10:58:42 18/5/2026</v>
+      </c>
+      <c r="O367" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P367" t="str">
+        <v>594</v>
+      </c>
+      <c r="Q367" t="str">
+        <v/>
+      </c>
+      <c r="R367" t="str">
+        <v/>
+      </c>
+      <c r="S367" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v/>
+      </c>
+      <c r="B368" t="str">
+        <v>Lu55_LU55_1_10</v>
+      </c>
+      <c r="C368" t="str">
+        <v>11,3068814</v>
+      </c>
+      <c r="D368" t="str">
+        <v>106,6366091</v>
+      </c>
+      <c r="E368" t="str">
+        <v/>
+      </c>
+      <c r="F368" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G368" t="str">
+        <v>3</v>
+      </c>
+      <c r="H368" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I368" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J368" t="str">
+        <v/>
+      </c>
+      <c r="K368" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L368" t="str">
+        <v>250</v>
+      </c>
+      <c r="M368" t="str">
+        <v/>
+      </c>
+      <c r="N368" t="str">
+        <v>10:58:48 18/5/2026</v>
+      </c>
+      <c r="O368" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P368" t="str">
+        <v>673</v>
+      </c>
+      <c r="Q368" t="str">
+        <v/>
+      </c>
+      <c r="R368" t="str">
+        <v/>
+      </c>
+      <c r="S368" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v/>
+      </c>
+      <c r="B369" t="str">
+        <v>Lu55_LU55_1_11</v>
+      </c>
+      <c r="C369" t="str">
+        <v>11,3067074</v>
+      </c>
+      <c r="D369" t="str">
+        <v>106,6372177</v>
+      </c>
+      <c r="E369" t="str">
+        <v/>
+      </c>
+      <c r="F369" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G369" t="str">
+        <v>3</v>
+      </c>
+      <c r="H369" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I369" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J369" t="str">
+        <v/>
+      </c>
+      <c r="K369" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L369" t="str">
+        <v>250</v>
+      </c>
+      <c r="M369" t="str">
+        <v/>
+      </c>
+      <c r="N369" t="str">
+        <v>11:00:55 18/5/2026</v>
+      </c>
+      <c r="O369" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P369" t="str">
+        <v>653</v>
+      </c>
+      <c r="Q369" t="str">
+        <v/>
+      </c>
+      <c r="R369" t="str">
+        <v>Quốc lộ 13</v>
+      </c>
+      <c r="S369" t="str">
+        <v>Xà Mách</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v/>
+      </c>
+      <c r="B370" t="str">
+        <v>Lu55_LU55_1_12</v>
+      </c>
+      <c r="C370" t="str">
+        <v>11,3065322</v>
+      </c>
+      <c r="D370" t="str">
+        <v>106,6377662</v>
+      </c>
+      <c r="E370" t="str">
+        <v/>
+      </c>
+      <c r="F370" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G370" t="str">
+        <v>3</v>
+      </c>
+      <c r="H370" t="str">
+        <v>Lai Uyên 55_1</v>
+      </c>
+      <c r="I370" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J370" t="str">
+        <v/>
+      </c>
+      <c r="K370" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L370" t="str">
+        <v>250</v>
+      </c>
+      <c r="M370" t="str">
+        <v/>
+      </c>
+      <c r="N370" t="str">
+        <v>11:00:56 18/5/2026</v>
+      </c>
+      <c r="O370" t="str">
+        <v>Lu55_LU55_1_1</v>
+      </c>
+      <c r="P370" t="str">
+        <v>819</v>
+      </c>
+      <c r="Q370" t="str">
+        <v/>
+      </c>
+      <c r="R370" t="str">
+        <v/>
+      </c>
+      <c r="S370" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v/>
+      </c>
+      <c r="B371" t="str">
+        <v>Lai uyên - 61_2</v>
+      </c>
+      <c r="C371" t="str">
+        <v>11,2938119</v>
+      </c>
+      <c r="D371" t="str">
+        <v>106,6364604</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Xã Bàu Bàng, Thành phố Hồ Chí Minh, 75751, Việt Nam</v>
+      </c>
+      <c r="F371" t="str">
+        <v>Nguyễn Trần Hiếu Nghĩa</v>
+      </c>
+      <c r="G371" t="str">
+        <v>6</v>
+      </c>
+      <c r="H371" t="str">
+        <v>101.240.000</v>
+      </c>
+      <c r="I371" t="str">
+        <v>Tủ chiếu sáng ngầm</v>
+      </c>
+      <c r="J371" t="str">
+        <v/>
+      </c>
+      <c r="K371" t="str">
+        <v/>
+      </c>
+      <c r="L371" t="str">
+        <v/>
+      </c>
+      <c r="M371" t="str">
+        <v/>
+      </c>
+      <c r="N371" t="str">
+        <v>08:44:09 19/5/2026</v>
+      </c>
+      <c r="O371" t="str">
+        <v>Lai uyên - 61_1</v>
+      </c>
+      <c r="P371" t="str">
+        <v/>
+      </c>
+      <c r="Q371" t="str">
+        <v/>
+      </c>
+      <c r="R371" t="str">
+        <v/>
+      </c>
+      <c r="S371" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v/>
+      </c>
+      <c r="B372" t="str">
+        <v>Lai Uyên-61_1</v>
+      </c>
+      <c r="C372" t="str">
+        <v>11,2940354</v>
+      </c>
+      <c r="D372" t="str">
+        <v>106,6325520</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Xã Bàu Bàng, Thành phố Hồ Chí Minh, 75751, Việt Nam</v>
+      </c>
+      <c r="F372" t="str">
+        <v>Nguyễn Trần Hiếu Nghĩa</v>
+      </c>
+      <c r="G372" t="str">
+        <v>6</v>
+      </c>
+      <c r="H372" t="str">
+        <v>101.241.000</v>
+      </c>
+      <c r="I372" t="str">
+        <v>Tủ chiếu sáng ngầm</v>
+      </c>
+      <c r="J372" t="str">
+        <v/>
+      </c>
+      <c r="K372" t="str">
+        <v/>
+      </c>
+      <c r="L372" t="str">
+        <v/>
+      </c>
+      <c r="M372" t="str">
+        <v/>
+      </c>
+      <c r="N372" t="str">
+        <v>08:45:35 19/5/2026</v>
+      </c>
+      <c r="O372" t="str">
+        <v/>
+      </c>
+      <c r="P372" t="str">
+        <v/>
+      </c>
+      <c r="Q372" t="str">
+        <v/>
+      </c>
+      <c r="R372" t="str">
+        <v/>
+      </c>
+      <c r="S372" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S358"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S372"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Đồng bộ dữ liệu khảo sát 2026-06-11
</commit_message>
<xml_diff>
--- a/data/khaosat.xlsx
+++ b/data/khaosat.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S372"/>
+  <dimension ref="A1:S419"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22347,9 +22347,2782 @@
         <v/>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v/>
+      </c>
+      <c r="B373" t="str">
+        <v>Lai Uyên 80-2</v>
+      </c>
+      <c r="C373" t="str">
+        <v>11,2867935</v>
+      </c>
+      <c r="D373" t="str">
+        <v>106,6376391</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Đường tỉnh 741C, Bến Lớn, Xã Bàu Bàng, Thành phố Hồ Chí Minh, 75751, Việt Nam</v>
+      </c>
+      <c r="F373" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G373" t="str">
+        <v>6</v>
+      </c>
+      <c r="H373" t="str">
+        <v>101.298.000</v>
+      </c>
+      <c r="I373" t="str">
+        <v>Tủ chiếu sáng ngầm</v>
+      </c>
+      <c r="J373" t="str">
+        <v/>
+      </c>
+      <c r="K373" t="str">
+        <v/>
+      </c>
+      <c r="L373" t="str">
+        <v/>
+      </c>
+      <c r="M373" t="str">
+        <v/>
+      </c>
+      <c r="N373" t="str">
+        <v>11:21:18 21/5/2026</v>
+      </c>
+      <c r="O373" t="str">
+        <v>Lai Uyên 80-2</v>
+      </c>
+      <c r="P373" t="str">
+        <v>2230</v>
+      </c>
+      <c r="Q373" t="str">
+        <v/>
+      </c>
+      <c r="R373" t="str">
+        <v>Đường tỉnh 741C</v>
+      </c>
+      <c r="S373" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v/>
+      </c>
+      <c r="B374" t="str">
+        <v>Lai Uyên 80-1</v>
+      </c>
+      <c r="C374" t="str">
+        <v>11,2841906</v>
+      </c>
+      <c r="D374" t="str">
+        <v>106,6579154</v>
+      </c>
+      <c r="E374" t="str">
+        <v>Phường Bến Cát, Thành phố Hồ Chí Minh, 75751, Việt Nam</v>
+      </c>
+      <c r="F374" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G374" t="str">
+        <v>5</v>
+      </c>
+      <c r="H374" t="str">
+        <v>101.144.000</v>
+      </c>
+      <c r="I374" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J374" t="str">
+        <v/>
+      </c>
+      <c r="K374" t="str">
+        <v/>
+      </c>
+      <c r="L374" t="str">
+        <v/>
+      </c>
+      <c r="M374" t="str">
+        <v/>
+      </c>
+      <c r="N374" t="str">
+        <v>11:21:46 21/5/2026</v>
+      </c>
+      <c r="O374" t="str">
+        <v>Lai Uyên 80-2</v>
+      </c>
+      <c r="P374" t="str">
+        <v/>
+      </c>
+      <c r="Q374" t="str">
+        <v/>
+      </c>
+      <c r="R374" t="str">
+        <v/>
+      </c>
+      <c r="S374" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v/>
+      </c>
+      <c r="B375" t="str">
+        <v>LU103_LU103_1</v>
+      </c>
+      <c r="C375" t="str">
+        <v>11,3053360</v>
+      </c>
+      <c r="D375" t="str">
+        <v>106,6630944</v>
+      </c>
+      <c r="E375" t="str">
+        <v/>
+      </c>
+      <c r="F375" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G375" t="str">
+        <v>3</v>
+      </c>
+      <c r="H375" t="str">
+        <v>Lai Uyên 103</v>
+      </c>
+      <c r="I375" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J375" t="str">
+        <v/>
+      </c>
+      <c r="K375" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L375" t="str">
+        <v/>
+      </c>
+      <c r="M375" t="str">
+        <v/>
+      </c>
+      <c r="N375" t="str">
+        <v>11:26:50 23/5/2026</v>
+      </c>
+      <c r="O375" t="str">
+        <v/>
+      </c>
+      <c r="P375" t="str">
+        <v/>
+      </c>
+      <c r="Q375" t="str">
+        <v>No25091916</v>
+      </c>
+      <c r="R375" t="str">
+        <v/>
+      </c>
+      <c r="S375" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v/>
+      </c>
+      <c r="B376" t="str">
+        <v>TĐK : Lai Uyên 103</v>
+      </c>
+      <c r="C376" t="str">
+        <v>11,3053212</v>
+      </c>
+      <c r="D376" t="str">
+        <v>106,6630964</v>
+      </c>
+      <c r="E376" t="str">
+        <v/>
+      </c>
+      <c r="F376" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G376" t="str">
+        <v>5</v>
+      </c>
+      <c r="H376" t="str">
+        <v>Lai Uyên 103</v>
+      </c>
+      <c r="I376" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J376" t="str">
+        <v/>
+      </c>
+      <c r="K376" t="str">
+        <v/>
+      </c>
+      <c r="L376" t="str">
+        <v/>
+      </c>
+      <c r="M376" t="str">
+        <v/>
+      </c>
+      <c r="N376" t="str">
+        <v>11:26:55 23/5/2026</v>
+      </c>
+      <c r="O376" t="str">
+        <v/>
+      </c>
+      <c r="P376" t="str">
+        <v/>
+      </c>
+      <c r="Q376" t="str">
+        <v>No25091916</v>
+      </c>
+      <c r="R376" t="str">
+        <v>Lai Uyên 103</v>
+      </c>
+      <c r="S376" t="str">
+        <v>Xã Bàu Bàng</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v/>
+      </c>
+      <c r="B377" t="str">
+        <v>LU13_LU13_11</v>
+      </c>
+      <c r="C377" t="str">
+        <v>11,3371892</v>
+      </c>
+      <c r="D377" t="str">
+        <v>106,6371673</v>
+      </c>
+      <c r="E377" t="str">
+        <v/>
+      </c>
+      <c r="F377" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G377" t="str">
+        <v>3</v>
+      </c>
+      <c r="H377" t="str">
+        <v>Lai Uyên 13</v>
+      </c>
+      <c r="I377" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J377" t="str">
+        <v/>
+      </c>
+      <c r="K377" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L377" t="str">
+        <v/>
+      </c>
+      <c r="M377" t="str">
+        <v/>
+      </c>
+      <c r="N377" t="str">
+        <v>12:48:32 23/5/2026</v>
+      </c>
+      <c r="O377" t="str">
+        <v/>
+      </c>
+      <c r="P377" t="str">
+        <v/>
+      </c>
+      <c r="Q377" t="str">
+        <v>No:2020088322</v>
+      </c>
+      <c r="R377" t="str">
+        <v>Lai Uyên 13</v>
+      </c>
+      <c r="S377" t="str">
+        <v>Khu phố Bàu Lòng</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v/>
+      </c>
+      <c r="B378" t="str">
+        <v>Lai Uyên ? Trụ 4</v>
+      </c>
+      <c r="C378" t="str">
+        <v>11,3387229</v>
+      </c>
+      <c r="D378" t="str">
+        <v>106,6427971</v>
+      </c>
+      <c r="E378" t="str">
+        <v/>
+      </c>
+      <c r="F378" t="str">
+        <v>Nguyễn Trần Hiếu Nghĩa</v>
+      </c>
+      <c r="G378" t="str">
+        <v>3</v>
+      </c>
+      <c r="H378" t="str">
+        <v>Lai Uyên?</v>
+      </c>
+      <c r="I378" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J378" t="str">
+        <v/>
+      </c>
+      <c r="K378" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L378" t="str">
+        <v/>
+      </c>
+      <c r="M378" t="str">
+        <v/>
+      </c>
+      <c r="N378" t="str">
+        <v>12:54:46 23/5/2026</v>
+      </c>
+      <c r="O378" t="str">
+        <v/>
+      </c>
+      <c r="P378" t="str">
+        <v/>
+      </c>
+      <c r="Q378" t="str">
+        <v>No.21065930</v>
+      </c>
+      <c r="R378" t="str">
+        <v/>
+      </c>
+      <c r="S378" t="str">
+        <v>Khu phố Bàu Lòng</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v/>
+      </c>
+      <c r="B379" t="str">
+        <v>LU17_LU17-T2_1</v>
+      </c>
+      <c r="C379" t="str">
+        <v>11,3315001</v>
+      </c>
+      <c r="D379" t="str">
+        <v>106,6334428</v>
+      </c>
+      <c r="E379" t="str">
+        <v/>
+      </c>
+      <c r="F379" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G379" t="str">
+        <v>4</v>
+      </c>
+      <c r="H379" t="str">
+        <v>LU17-T2</v>
+      </c>
+      <c r="I379" t="str">
+        <v>Trụ TTLT</v>
+      </c>
+      <c r="J379" t="str">
+        <v/>
+      </c>
+      <c r="K379" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L379" t="str">
+        <v/>
+      </c>
+      <c r="M379" t="str">
+        <v/>
+      </c>
+      <c r="N379" t="str">
+        <v>14:00:54 23/5/2026</v>
+      </c>
+      <c r="O379" t="str">
+        <v/>
+      </c>
+      <c r="P379" t="str">
+        <v/>
+      </c>
+      <c r="Q379" t="str">
+        <v>No:25088063</v>
+      </c>
+      <c r="R379" t="str">
+        <v/>
+      </c>
+      <c r="S379" t="str">
+        <v>Khu phố Bàu Lòng</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v/>
+      </c>
+      <c r="B380" t="str">
+        <v>TĐK: ĐH618-3</v>
+      </c>
+      <c r="C380" t="str">
+        <v>11,3073415</v>
+      </c>
+      <c r="D380" t="str">
+        <v>106,6622244</v>
+      </c>
+      <c r="E380" t="str">
+        <v/>
+      </c>
+      <c r="F380" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G380" t="str">
+        <v>5</v>
+      </c>
+      <c r="H380" t="str">
+        <v>ĐH618-3</v>
+      </c>
+      <c r="I380" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J380" t="str">
+        <v/>
+      </c>
+      <c r="K380" t="str">
+        <v/>
+      </c>
+      <c r="L380" t="str">
+        <v/>
+      </c>
+      <c r="M380" t="str">
+        <v/>
+      </c>
+      <c r="N380" t="str">
+        <v>15:00:25 23/5/2026</v>
+      </c>
+      <c r="O380" t="str">
+        <v/>
+      </c>
+      <c r="P380" t="str">
+        <v/>
+      </c>
+      <c r="Q380" t="str">
+        <v>No.1511225119</v>
+      </c>
+      <c r="R380" t="str">
+        <v/>
+      </c>
+      <c r="S380" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v/>
+      </c>
+      <c r="B381" t="str">
+        <v>TĐK: ĐH618-4</v>
+      </c>
+      <c r="C381" t="str">
+        <v>11,3109099</v>
+      </c>
+      <c r="D381" t="str">
+        <v>106,6544889</v>
+      </c>
+      <c r="E381" t="str">
+        <v/>
+      </c>
+      <c r="F381" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G381" t="str">
+        <v>5</v>
+      </c>
+      <c r="H381" t="str">
+        <v>ĐH618-4</v>
+      </c>
+      <c r="I381" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J381" t="str">
+        <v/>
+      </c>
+      <c r="K381" t="str">
+        <v/>
+      </c>
+      <c r="L381" t="str">
+        <v/>
+      </c>
+      <c r="M381" t="str">
+        <v/>
+      </c>
+      <c r="N381" t="str">
+        <v>15:02:17 23/5/2026</v>
+      </c>
+      <c r="O381" t="str">
+        <v>TĐK: ĐH618-3</v>
+      </c>
+      <c r="P381" t="str">
+        <v>930</v>
+      </c>
+      <c r="Q381" t="str">
+        <v>No.1511025355</v>
+      </c>
+      <c r="R381" t="str">
+        <v/>
+      </c>
+      <c r="S381" t="str">
+        <v>Bến Lớn</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v/>
+      </c>
+      <c r="B382" t="str">
+        <v>TĐK: ĐH618-5</v>
+      </c>
+      <c r="C382" t="str">
+        <v>11,3179717</v>
+      </c>
+      <c r="D382" t="str">
+        <v>106,6412643</v>
+      </c>
+      <c r="E382" t="str">
+        <v/>
+      </c>
+      <c r="F382" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G382" t="str">
+        <v>5</v>
+      </c>
+      <c r="H382" t="str">
+        <v>ĐH618-5</v>
+      </c>
+      <c r="I382" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J382" t="str">
+        <v/>
+      </c>
+      <c r="K382" t="str">
+        <v/>
+      </c>
+      <c r="L382" t="str">
+        <v/>
+      </c>
+      <c r="M382" t="str">
+        <v/>
+      </c>
+      <c r="N382" t="str">
+        <v>15:04:04 23/5/2026</v>
+      </c>
+      <c r="O382" t="str">
+        <v>TĐK: ĐH618-3</v>
+      </c>
+      <c r="P382" t="str">
+        <v>2586</v>
+      </c>
+      <c r="Q382" t="str">
+        <v>No.1511025355</v>
+      </c>
+      <c r="R382" t="str">
+        <v/>
+      </c>
+      <c r="S382" t="str">
+        <v>Bàu Hốt</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v/>
+      </c>
+      <c r="B383" t="str">
+        <v>TĐK: Lai Uyên 15-T1</v>
+      </c>
+      <c r="C383" t="str">
+        <v>11,3349652</v>
+      </c>
+      <c r="D383" t="str">
+        <v>106,6368990</v>
+      </c>
+      <c r="E383" t="str">
+        <v/>
+      </c>
+      <c r="F383" t="str">
+        <v>Phạm Văn Tính</v>
+      </c>
+      <c r="G383" t="str">
+        <v>5</v>
+      </c>
+      <c r="H383" t="str">
+        <v>Lai Uyên 15-T1</v>
+      </c>
+      <c r="I383" t="str">
+        <v>Tủ chiếu sáng nổi</v>
+      </c>
+      <c r="J383" t="str">
+        <v/>
+      </c>
+      <c r="K383" t="str">
+        <v/>
+      </c>
+      <c r="L383" t="str">
+        <v/>
+      </c>
+      <c r="M383" t="str">
+        <v/>
+      </c>
+      <c r="N383" t="str">
+        <v>15:07:20 23/5/2026</v>
+      </c>
+      <c r="O383" t="str">
+        <v/>
+      </c>
+      <c r="P383" t="str">
+        <v/>
+      </c>
+      <c r="Q383" t="str">
+        <v>No:2020214453</v>
+      </c>
+      <c r="R383" t="str">
+        <v>Quốc lộ 13</v>
+      </c>
+      <c r="S383" t="str">
+        <v>Xà Mách</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v/>
+      </c>
+      <c r="B384" t="str">
+        <v>LU_LU15_7</v>
+      </c>
+      <c r="C384" t="str">
+        <v>11,3347798</v>
+      </c>
+      <c r="D384" t="str">
+        <v>106,6369070</v>
+      </c>
+      <c r="E384" t="str">
+        <v/>
+      </c>
+      <c r="F384" t="str">
+        <v>Nguyễn Quí Tiên</v>
+      </c>
+      <c r="G384" t="str">
+        <v>3</v>
+      </c>
+      <c r="H384" t="str">
+        <v>Lai Uyên 15-T ?</v>
+      </c>
+      <c r="I384" t="str">
+        <v>Trụ HTLT</v>
+      </c>
+      <c r="J384" t="str">
+        <v/>
+      </c>
+      <c r="K384" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L384" t="str">
+        <v/>
+      </c>
+      <c r="M384" t="str">
+        <v/>
+      </c>
+      <c r="N384" t="str">
+        <v>15:06:22 23/5/2026</v>
+      </c>
+      <c r="O384" t="str">
+        <v/>
+      </c>
+      <c r="P384" t="str">
+        <v/>
+      </c>
+      <c r="Q384" t="str">
+        <v>No:2020214453</v>
+      </c>
+      <c r="R384" t="str">
+        <v>Lai Uyên 15</v>
+      </c>
+      <c r="S384" t="str">
+        <v>Xà Mách</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v/>
+      </c>
+      <c r="B385" t="str">
+        <v>VTS_H232VTS_1</v>
+      </c>
+      <c r="C385" t="str">
+        <v>10,7844640</v>
+      </c>
+      <c r="D385" t="str">
+        <v>106,6884939</v>
+      </c>
+      <c r="E385" t="str">
+        <v/>
+      </c>
+      <c r="F385" t="str">
+        <v/>
+      </c>
+      <c r="G385" t="str">
+        <v>1</v>
+      </c>
+      <c r="H385" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I385" t="str">
+        <v/>
+      </c>
+      <c r="J385" t="str">
+        <v/>
+      </c>
+      <c r="K385" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L385" t="str">
+        <v/>
+      </c>
+      <c r="M385" t="str">
+        <v/>
+      </c>
+      <c r="N385" t="str">
+        <v>11:31:47 11/6/2026</v>
+      </c>
+      <c r="O385" t="str">
+        <v/>
+      </c>
+      <c r="P385" t="str">
+        <v/>
+      </c>
+      <c r="Q385" t="str">
+        <v/>
+      </c>
+      <c r="R385" t="str">
+        <v/>
+      </c>
+      <c r="S385" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v/>
+      </c>
+      <c r="B386" t="str">
+        <v>VTS_H232VTS_2</v>
+      </c>
+      <c r="C386" t="str">
+        <v>10,7842111</v>
+      </c>
+      <c r="D386" t="str">
+        <v>106,6882123</v>
+      </c>
+      <c r="E386" t="str">
+        <v/>
+      </c>
+      <c r="F386" t="str">
+        <v/>
+      </c>
+      <c r="G386" t="str">
+        <v>1</v>
+      </c>
+      <c r="H386" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I386" t="str">
+        <v/>
+      </c>
+      <c r="J386" t="str">
+        <v/>
+      </c>
+      <c r="K386" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L386" t="str">
+        <v/>
+      </c>
+      <c r="M386" t="str">
+        <v/>
+      </c>
+      <c r="N386" t="str">
+        <v>11:31:40 11/6/2026</v>
+      </c>
+      <c r="O386" t="str">
+        <v>VTS_H232VTS_1</v>
+      </c>
+      <c r="P386" t="str">
+        <v/>
+      </c>
+      <c r="Q386" t="str">
+        <v/>
+      </c>
+      <c r="R386" t="str">
+        <v/>
+      </c>
+      <c r="S386" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v/>
+      </c>
+      <c r="B387" t="str">
+        <v>VTS_H232VTS_3</v>
+      </c>
+      <c r="C387" t="str">
+        <v>10,7840293</v>
+      </c>
+      <c r="D387" t="str">
+        <v>106,6880420</v>
+      </c>
+      <c r="E387" t="str">
+        <v/>
+      </c>
+      <c r="F387" t="str">
+        <v/>
+      </c>
+      <c r="G387" t="str">
+        <v>1</v>
+      </c>
+      <c r="H387" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I387" t="str">
+        <v/>
+      </c>
+      <c r="J387" t="str">
+        <v/>
+      </c>
+      <c r="K387" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L387" t="str">
+        <v/>
+      </c>
+      <c r="M387" t="str">
+        <v/>
+      </c>
+      <c r="N387" t="str">
+        <v>11:32:31 11/6/2026</v>
+      </c>
+      <c r="O387" t="str">
+        <v>VTS_H232VTS_2</v>
+      </c>
+      <c r="P387" t="str">
+        <v/>
+      </c>
+      <c r="Q387" t="str">
+        <v/>
+      </c>
+      <c r="R387" t="str">
+        <v/>
+      </c>
+      <c r="S387" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v/>
+      </c>
+      <c r="B388" t="str">
+        <v>VTS_H232VTS_4</v>
+      </c>
+      <c r="C388" t="str">
+        <v>10,7837882</v>
+      </c>
+      <c r="D388" t="str">
+        <v>106,6877979</v>
+      </c>
+      <c r="E388" t="str">
+        <v/>
+      </c>
+      <c r="F388" t="str">
+        <v/>
+      </c>
+      <c r="G388" t="str">
+        <v>1</v>
+      </c>
+      <c r="H388" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I388" t="str">
+        <v/>
+      </c>
+      <c r="J388" t="str">
+        <v/>
+      </c>
+      <c r="K388" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L388" t="str">
+        <v/>
+      </c>
+      <c r="M388" t="str">
+        <v/>
+      </c>
+      <c r="N388" t="str">
+        <v>11:32:28 11/6/2026</v>
+      </c>
+      <c r="O388" t="str">
+        <v>VTS_H232VTS_3</v>
+      </c>
+      <c r="P388" t="str">
+        <v/>
+      </c>
+      <c r="Q388" t="str">
+        <v/>
+      </c>
+      <c r="R388" t="str">
+        <v/>
+      </c>
+      <c r="S388" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v/>
+      </c>
+      <c r="B389" t="str">
+        <v>VTS_H232VTS_5</v>
+      </c>
+      <c r="C389" t="str">
+        <v>10,7835399</v>
+      </c>
+      <c r="D389" t="str">
+        <v>106,6876055</v>
+      </c>
+      <c r="E389" t="str">
+        <v/>
+      </c>
+      <c r="F389" t="str">
+        <v/>
+      </c>
+      <c r="G389" t="str">
+        <v>1</v>
+      </c>
+      <c r="H389" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I389" t="str">
+        <v/>
+      </c>
+      <c r="J389" t="str">
+        <v/>
+      </c>
+      <c r="K389" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L389" t="str">
+        <v/>
+      </c>
+      <c r="M389" t="str">
+        <v/>
+      </c>
+      <c r="N389" t="str">
+        <v>11:30:18 11/6/2026</v>
+      </c>
+      <c r="O389" t="str">
+        <v>VTS_H232VTS_4</v>
+      </c>
+      <c r="P389" t="str">
+        <v/>
+      </c>
+      <c r="Q389" t="str">
+        <v/>
+      </c>
+      <c r="R389" t="str">
+        <v/>
+      </c>
+      <c r="S389" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v/>
+      </c>
+      <c r="B390" t="str">
+        <v>VTS_H232VTS_6</v>
+      </c>
+      <c r="C390" t="str">
+        <v>10,7831980</v>
+      </c>
+      <c r="D390" t="str">
+        <v>106,6872387</v>
+      </c>
+      <c r="E390" t="str">
+        <v/>
+      </c>
+      <c r="F390" t="str">
+        <v/>
+      </c>
+      <c r="G390" t="str">
+        <v>1</v>
+      </c>
+      <c r="H390" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I390" t="str">
+        <v/>
+      </c>
+      <c r="J390" t="str">
+        <v/>
+      </c>
+      <c r="K390" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L390" t="str">
+        <v/>
+      </c>
+      <c r="M390" t="str">
+        <v/>
+      </c>
+      <c r="N390" t="str">
+        <v>11:32:06 11/6/2026</v>
+      </c>
+      <c r="O390" t="str">
+        <v>VTS_H232VTS_5</v>
+      </c>
+      <c r="P390" t="str">
+        <v/>
+      </c>
+      <c r="Q390" t="str">
+        <v/>
+      </c>
+      <c r="R390" t="str">
+        <v/>
+      </c>
+      <c r="S390" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v/>
+      </c>
+      <c r="B391" t="str">
+        <v>VTS_H232VTS_7</v>
+      </c>
+      <c r="C391" t="str">
+        <v>10,7833416</v>
+      </c>
+      <c r="D391" t="str">
+        <v>106,6873848</v>
+      </c>
+      <c r="E391" t="str">
+        <v/>
+      </c>
+      <c r="F391" t="str">
+        <v/>
+      </c>
+      <c r="G391" t="str">
+        <v>1</v>
+      </c>
+      <c r="H391" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I391" t="str">
+        <v/>
+      </c>
+      <c r="J391" t="str">
+        <v/>
+      </c>
+      <c r="K391" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L391" t="str">
+        <v/>
+      </c>
+      <c r="M391" t="str">
+        <v/>
+      </c>
+      <c r="N391" t="str">
+        <v>11:32:02 11/6/2026</v>
+      </c>
+      <c r="O391" t="str">
+        <v>VTS_H232VTS_6</v>
+      </c>
+      <c r="P391" t="str">
+        <v/>
+      </c>
+      <c r="Q391" t="str">
+        <v/>
+      </c>
+      <c r="R391" t="str">
+        <v/>
+      </c>
+      <c r="S391" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v/>
+      </c>
+      <c r="B392" t="str">
+        <v>VTS_H232VTS_8</v>
+      </c>
+      <c r="C392" t="str">
+        <v>10,7830452</v>
+      </c>
+      <c r="D392" t="str">
+        <v>106,6870911</v>
+      </c>
+      <c r="E392" t="str">
+        <v/>
+      </c>
+      <c r="F392" t="str">
+        <v/>
+      </c>
+      <c r="G392" t="str">
+        <v>1</v>
+      </c>
+      <c r="H392" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I392" t="str">
+        <v/>
+      </c>
+      <c r="J392" t="str">
+        <v/>
+      </c>
+      <c r="K392" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L392" t="str">
+        <v/>
+      </c>
+      <c r="M392" t="str">
+        <v/>
+      </c>
+      <c r="N392" t="str">
+        <v>11:32:15 11/6/2026</v>
+      </c>
+      <c r="O392" t="str">
+        <v>VTS_H232VTS_7</v>
+      </c>
+      <c r="P392" t="str">
+        <v/>
+      </c>
+      <c r="Q392" t="str">
+        <v/>
+      </c>
+      <c r="R392" t="str">
+        <v/>
+      </c>
+      <c r="S392" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v/>
+      </c>
+      <c r="B393" t="str">
+        <v>VTS_H232VTS_9</v>
+      </c>
+      <c r="C393" t="str">
+        <v>10,7828410</v>
+      </c>
+      <c r="D393" t="str">
+        <v>106,6868967</v>
+      </c>
+      <c r="E393" t="str">
+        <v/>
+      </c>
+      <c r="F393" t="str">
+        <v/>
+      </c>
+      <c r="G393" t="str">
+        <v>1</v>
+      </c>
+      <c r="H393" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I393" t="str">
+        <v/>
+      </c>
+      <c r="J393" t="str">
+        <v/>
+      </c>
+      <c r="K393" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L393" t="str">
+        <v/>
+      </c>
+      <c r="M393" t="str">
+        <v/>
+      </c>
+      <c r="N393" t="str">
+        <v>11:32:12 11/6/2026</v>
+      </c>
+      <c r="O393" t="str">
+        <v>VTS_H232VTS_8</v>
+      </c>
+      <c r="P393" t="str">
+        <v/>
+      </c>
+      <c r="Q393" t="str">
+        <v/>
+      </c>
+      <c r="R393" t="str">
+        <v/>
+      </c>
+      <c r="S393" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v/>
+      </c>
+      <c r="B394" t="str">
+        <v>VTS_H232VTS_10</v>
+      </c>
+      <c r="C394" t="str">
+        <v>10,7826631</v>
+      </c>
+      <c r="D394" t="str">
+        <v>106,6867223</v>
+      </c>
+      <c r="E394" t="str">
+        <v/>
+      </c>
+      <c r="F394" t="str">
+        <v/>
+      </c>
+      <c r="G394" t="str">
+        <v>1</v>
+      </c>
+      <c r="H394" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I394" t="str">
+        <v/>
+      </c>
+      <c r="J394" t="str">
+        <v/>
+      </c>
+      <c r="K394" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L394" t="str">
+        <v/>
+      </c>
+      <c r="M394" t="str">
+        <v/>
+      </c>
+      <c r="N394" t="str">
+        <v>11:32:23 11/6/2026</v>
+      </c>
+      <c r="O394" t="str">
+        <v>VTS_H232VTS_9</v>
+      </c>
+      <c r="P394" t="str">
+        <v/>
+      </c>
+      <c r="Q394" t="str">
+        <v/>
+      </c>
+      <c r="R394" t="str">
+        <v/>
+      </c>
+      <c r="S394" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v/>
+      </c>
+      <c r="B395" t="str">
+        <v>VTS_H232VTS_11</v>
+      </c>
+      <c r="C395" t="str">
+        <v>10,7825235</v>
+      </c>
+      <c r="D395" t="str">
+        <v>106,6865788</v>
+      </c>
+      <c r="E395" t="str">
+        <v/>
+      </c>
+      <c r="F395" t="str">
+        <v/>
+      </c>
+      <c r="G395" t="str">
+        <v>1</v>
+      </c>
+      <c r="H395" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I395" t="str">
+        <v/>
+      </c>
+      <c r="J395" t="str">
+        <v/>
+      </c>
+      <c r="K395" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L395" t="str">
+        <v/>
+      </c>
+      <c r="M395" t="str">
+        <v/>
+      </c>
+      <c r="N395" t="str">
+        <v>11:32:17 11/6/2026</v>
+      </c>
+      <c r="O395" t="str">
+        <v>VTS_H232VTS_10</v>
+      </c>
+      <c r="P395" t="str">
+        <v/>
+      </c>
+      <c r="Q395" t="str">
+        <v/>
+      </c>
+      <c r="R395" t="str">
+        <v/>
+      </c>
+      <c r="S395" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v/>
+      </c>
+      <c r="B396" t="str">
+        <v>VTS_H232VTS_12</v>
+      </c>
+      <c r="C396" t="str">
+        <v>10,7823796</v>
+      </c>
+      <c r="D396" t="str">
+        <v>106,6864128</v>
+      </c>
+      <c r="E396" t="str">
+        <v/>
+      </c>
+      <c r="F396" t="str">
+        <v/>
+      </c>
+      <c r="G396" t="str">
+        <v>1</v>
+      </c>
+      <c r="H396" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I396" t="str">
+        <v/>
+      </c>
+      <c r="J396" t="str">
+        <v/>
+      </c>
+      <c r="K396" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L396" t="str">
+        <v/>
+      </c>
+      <c r="M396" t="str">
+        <v/>
+      </c>
+      <c r="N396" t="str">
+        <v>11:15:15 11/6/2026</v>
+      </c>
+      <c r="O396" t="str">
+        <v>VTS_H232VTS_11</v>
+      </c>
+      <c r="P396" t="str">
+        <v/>
+      </c>
+      <c r="Q396" t="str">
+        <v/>
+      </c>
+      <c r="R396" t="str">
+        <v/>
+      </c>
+      <c r="S396" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v/>
+      </c>
+      <c r="B397" t="str">
+        <v>VTS_H232VTS_13</v>
+      </c>
+      <c r="C397" t="str">
+        <v>10,7821767</v>
+      </c>
+      <c r="D397" t="str">
+        <v>106,6862069</v>
+      </c>
+      <c r="E397" t="str">
+        <v/>
+      </c>
+      <c r="F397" t="str">
+        <v/>
+      </c>
+      <c r="G397" t="str">
+        <v>1</v>
+      </c>
+      <c r="H397" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I397" t="str">
+        <v/>
+      </c>
+      <c r="J397" t="str">
+        <v/>
+      </c>
+      <c r="K397" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L397" t="str">
+        <v/>
+      </c>
+      <c r="M397" t="str">
+        <v/>
+      </c>
+      <c r="N397" t="str">
+        <v>11:15:18 11/6/2026</v>
+      </c>
+      <c r="O397" t="str">
+        <v>VTS_H232VTS_12</v>
+      </c>
+      <c r="P397" t="str">
+        <v/>
+      </c>
+      <c r="Q397" t="str">
+        <v/>
+      </c>
+      <c r="R397" t="str">
+        <v/>
+      </c>
+      <c r="S397" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v/>
+      </c>
+      <c r="B398" t="str">
+        <v>VTS_H232VTS_14</v>
+      </c>
+      <c r="C398" t="str">
+        <v>10,7819395</v>
+      </c>
+      <c r="D398" t="str">
+        <v>106,6860202</v>
+      </c>
+      <c r="E398" t="str">
+        <v/>
+      </c>
+      <c r="F398" t="str">
+        <v/>
+      </c>
+      <c r="G398" t="str">
+        <v>1</v>
+      </c>
+      <c r="H398" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I398" t="str">
+        <v/>
+      </c>
+      <c r="J398" t="str">
+        <v/>
+      </c>
+      <c r="K398" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L398" t="str">
+        <v/>
+      </c>
+      <c r="M398" t="str">
+        <v/>
+      </c>
+      <c r="N398" t="str">
+        <v>11:15:20 11/6/2026</v>
+      </c>
+      <c r="O398" t="str">
+        <v>VTS_H232VTS_13</v>
+      </c>
+      <c r="P398" t="str">
+        <v/>
+      </c>
+      <c r="Q398" t="str">
+        <v/>
+      </c>
+      <c r="R398" t="str">
+        <v/>
+      </c>
+      <c r="S398" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v/>
+      </c>
+      <c r="B399" t="str">
+        <v>VTS_H232VTS_15</v>
+      </c>
+      <c r="C399" t="str">
+        <v>10,7816949</v>
+      </c>
+      <c r="D399" t="str">
+        <v>106,6857376</v>
+      </c>
+      <c r="E399" t="str">
+        <v/>
+      </c>
+      <c r="F399" t="str">
+        <v/>
+      </c>
+      <c r="G399" t="str">
+        <v>1</v>
+      </c>
+      <c r="H399" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I399" t="str">
+        <v/>
+      </c>
+      <c r="J399" t="str">
+        <v/>
+      </c>
+      <c r="K399" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L399" t="str">
+        <v/>
+      </c>
+      <c r="M399" t="str">
+        <v/>
+      </c>
+      <c r="N399" t="str">
+        <v>11:15:25 11/6/2026</v>
+      </c>
+      <c r="O399" t="str">
+        <v>VTS_H232VTS_14</v>
+      </c>
+      <c r="P399" t="str">
+        <v/>
+      </c>
+      <c r="Q399" t="str">
+        <v/>
+      </c>
+      <c r="R399" t="str">
+        <v/>
+      </c>
+      <c r="S399" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v/>
+      </c>
+      <c r="B400" t="str">
+        <v>VTS_H232VTS_16</v>
+      </c>
+      <c r="C400" t="str">
+        <v>10,7815237</v>
+      </c>
+      <c r="D400" t="str">
+        <v>106,6855774</v>
+      </c>
+      <c r="E400" t="str">
+        <v/>
+      </c>
+      <c r="F400" t="str">
+        <v/>
+      </c>
+      <c r="G400" t="str">
+        <v>1</v>
+      </c>
+      <c r="H400" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I400" t="str">
+        <v/>
+      </c>
+      <c r="J400" t="str">
+        <v/>
+      </c>
+      <c r="K400" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L400" t="str">
+        <v/>
+      </c>
+      <c r="M400" t="str">
+        <v/>
+      </c>
+      <c r="N400" t="str">
+        <v>11:15:28 11/6/2026</v>
+      </c>
+      <c r="O400" t="str">
+        <v>VTS_H232VTS_15</v>
+      </c>
+      <c r="P400" t="str">
+        <v/>
+      </c>
+      <c r="Q400" t="str">
+        <v/>
+      </c>
+      <c r="R400" t="str">
+        <v/>
+      </c>
+      <c r="S400" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v/>
+      </c>
+      <c r="B401" t="str">
+        <v>VTS_H232VTS_17</v>
+      </c>
+      <c r="C401" t="str">
+        <v>10,7813483</v>
+      </c>
+      <c r="D401" t="str">
+        <v>106,6854228</v>
+      </c>
+      <c r="E401" t="str">
+        <v/>
+      </c>
+      <c r="F401" t="str">
+        <v/>
+      </c>
+      <c r="G401" t="str">
+        <v>1</v>
+      </c>
+      <c r="H401" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I401" t="str">
+        <v/>
+      </c>
+      <c r="J401" t="str">
+        <v/>
+      </c>
+      <c r="K401" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L401" t="str">
+        <v/>
+      </c>
+      <c r="M401" t="str">
+        <v/>
+      </c>
+      <c r="N401" t="str">
+        <v>11:29:35 11/6/2026</v>
+      </c>
+      <c r="O401" t="str">
+        <v>VTS_H232VTS_16</v>
+      </c>
+      <c r="P401" t="str">
+        <v/>
+      </c>
+      <c r="Q401" t="str">
+        <v/>
+      </c>
+      <c r="R401" t="str">
+        <v/>
+      </c>
+      <c r="S401" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v/>
+      </c>
+      <c r="B402" t="str">
+        <v>VTS_H232VTS_18</v>
+      </c>
+      <c r="C402" t="str">
+        <v>10,7811362</v>
+      </c>
+      <c r="D402" t="str">
+        <v>106,6852055</v>
+      </c>
+      <c r="E402" t="str">
+        <v/>
+      </c>
+      <c r="F402" t="str">
+        <v/>
+      </c>
+      <c r="G402" t="str">
+        <v>1</v>
+      </c>
+      <c r="H402" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I402" t="str">
+        <v/>
+      </c>
+      <c r="J402" t="str">
+        <v/>
+      </c>
+      <c r="K402" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L402" t="str">
+        <v/>
+      </c>
+      <c r="M402" t="str">
+        <v/>
+      </c>
+      <c r="N402" t="str">
+        <v>11:29:33 11/6/2026</v>
+      </c>
+      <c r="O402" t="str">
+        <v>VTS_H232VTS_17</v>
+      </c>
+      <c r="P402" t="str">
+        <v/>
+      </c>
+      <c r="Q402" t="str">
+        <v/>
+      </c>
+      <c r="R402" t="str">
+        <v/>
+      </c>
+      <c r="S402" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v/>
+      </c>
+      <c r="B403" t="str">
+        <v>VTS_H232VTS_19</v>
+      </c>
+      <c r="C403" t="str">
+        <v>10,7809333</v>
+      </c>
+      <c r="D403" t="str">
+        <v>106,6849977</v>
+      </c>
+      <c r="E403" t="str">
+        <v/>
+      </c>
+      <c r="F403" t="str">
+        <v/>
+      </c>
+      <c r="G403" t="str">
+        <v>1</v>
+      </c>
+      <c r="H403" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I403" t="str">
+        <v/>
+      </c>
+      <c r="J403" t="str">
+        <v/>
+      </c>
+      <c r="K403" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L403" t="str">
+        <v/>
+      </c>
+      <c r="M403" t="str">
+        <v/>
+      </c>
+      <c r="N403" t="str">
+        <v>11:29:29 11/6/2026</v>
+      </c>
+      <c r="O403" t="str">
+        <v>VTS_H232VTS_18</v>
+      </c>
+      <c r="P403" t="str">
+        <v/>
+      </c>
+      <c r="Q403" t="str">
+        <v/>
+      </c>
+      <c r="R403" t="str">
+        <v/>
+      </c>
+      <c r="S403" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v/>
+      </c>
+      <c r="B404" t="str">
+        <v>VTS_H232VTS_20</v>
+      </c>
+      <c r="C404" t="str">
+        <v>10,7807094</v>
+      </c>
+      <c r="D404" t="str">
+        <v>106,6847670</v>
+      </c>
+      <c r="E404" t="str">
+        <v/>
+      </c>
+      <c r="F404" t="str">
+        <v/>
+      </c>
+      <c r="G404" t="str">
+        <v>1</v>
+      </c>
+      <c r="H404" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I404" t="str">
+        <v/>
+      </c>
+      <c r="J404" t="str">
+        <v/>
+      </c>
+      <c r="K404" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L404" t="str">
+        <v/>
+      </c>
+      <c r="M404" t="str">
+        <v/>
+      </c>
+      <c r="N404" t="str">
+        <v>11:29:09 11/6/2026</v>
+      </c>
+      <c r="O404" t="str">
+        <v>VTS_H232VTS_19</v>
+      </c>
+      <c r="P404" t="str">
+        <v/>
+      </c>
+      <c r="Q404" t="str">
+        <v/>
+      </c>
+      <c r="R404" t="str">
+        <v/>
+      </c>
+      <c r="S404" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v/>
+      </c>
+      <c r="B405" t="str">
+        <v>VTS_H232VTS_21</v>
+      </c>
+      <c r="C405" t="str">
+        <v>10,7805645</v>
+      </c>
+      <c r="D405" t="str">
+        <v>106,6846289</v>
+      </c>
+      <c r="E405" t="str">
+        <v/>
+      </c>
+      <c r="F405" t="str">
+        <v/>
+      </c>
+      <c r="G405" t="str">
+        <v>1</v>
+      </c>
+      <c r="H405" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I405" t="str">
+        <v/>
+      </c>
+      <c r="J405" t="str">
+        <v/>
+      </c>
+      <c r="K405" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L405" t="str">
+        <v/>
+      </c>
+      <c r="M405" t="str">
+        <v/>
+      </c>
+      <c r="N405" t="str">
+        <v>11:29:06 11/6/2026</v>
+      </c>
+      <c r="O405" t="str">
+        <v>VTS_H232VTS_20</v>
+      </c>
+      <c r="P405" t="str">
+        <v/>
+      </c>
+      <c r="Q405" t="str">
+        <v/>
+      </c>
+      <c r="R405" t="str">
+        <v/>
+      </c>
+      <c r="S405" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v/>
+      </c>
+      <c r="B406" t="str">
+        <v>VTS_H232VTS_22</v>
+      </c>
+      <c r="C406" t="str">
+        <v>10,7803994</v>
+      </c>
+      <c r="D406" t="str">
+        <v>106,6844508</v>
+      </c>
+      <c r="E406" t="str">
+        <v/>
+      </c>
+      <c r="F406" t="str">
+        <v/>
+      </c>
+      <c r="G406" t="str">
+        <v>1</v>
+      </c>
+      <c r="H406" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I406" t="str">
+        <v/>
+      </c>
+      <c r="J406" t="str">
+        <v/>
+      </c>
+      <c r="K406" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L406" t="str">
+        <v/>
+      </c>
+      <c r="M406" t="str">
+        <v/>
+      </c>
+      <c r="N406" t="str">
+        <v/>
+      </c>
+      <c r="O406" t="str">
+        <v>VTS_H232VTS_21</v>
+      </c>
+      <c r="P406" t="str">
+        <v/>
+      </c>
+      <c r="Q406" t="str">
+        <v/>
+      </c>
+      <c r="R406" t="str">
+        <v/>
+      </c>
+      <c r="S406" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v/>
+      </c>
+      <c r="B407" t="str">
+        <v>VTS_H232VTS_23</v>
+      </c>
+      <c r="C407" t="str">
+        <v>10,7801958</v>
+      </c>
+      <c r="D407" t="str">
+        <v>106,6842512</v>
+      </c>
+      <c r="E407" t="str">
+        <v/>
+      </c>
+      <c r="F407" t="str">
+        <v/>
+      </c>
+      <c r="G407" t="str">
+        <v>1</v>
+      </c>
+      <c r="H407" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I407" t="str">
+        <v/>
+      </c>
+      <c r="J407" t="str">
+        <v/>
+      </c>
+      <c r="K407" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L407" t="str">
+        <v/>
+      </c>
+      <c r="M407" t="str">
+        <v/>
+      </c>
+      <c r="N407" t="str">
+        <v>16:02:09 10/6/2026</v>
+      </c>
+      <c r="O407" t="str">
+        <v>VTS_H232VTS_22</v>
+      </c>
+      <c r="P407" t="str">
+        <v/>
+      </c>
+      <c r="Q407" t="str">
+        <v/>
+      </c>
+      <c r="R407" t="str">
+        <v/>
+      </c>
+      <c r="S407" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v/>
+      </c>
+      <c r="B408" t="str">
+        <v>VTS_H232VTS_24</v>
+      </c>
+      <c r="C408" t="str">
+        <v>10,7799776</v>
+      </c>
+      <c r="D408" t="str">
+        <v>106,6840352</v>
+      </c>
+      <c r="E408" t="str">
+        <v/>
+      </c>
+      <c r="F408" t="str">
+        <v/>
+      </c>
+      <c r="G408" t="str">
+        <v>1</v>
+      </c>
+      <c r="H408" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I408" t="str">
+        <v/>
+      </c>
+      <c r="J408" t="str">
+        <v/>
+      </c>
+      <c r="K408" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L408" t="str">
+        <v/>
+      </c>
+      <c r="M408" t="str">
+        <v/>
+      </c>
+      <c r="N408" t="str">
+        <v/>
+      </c>
+      <c r="O408" t="str">
+        <v>VTS_H232VTS_23</v>
+      </c>
+      <c r="P408" t="str">
+        <v/>
+      </c>
+      <c r="Q408" t="str">
+        <v/>
+      </c>
+      <c r="R408" t="str">
+        <v/>
+      </c>
+      <c r="S408" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v/>
+      </c>
+      <c r="B409" t="str">
+        <v>VTS_H232VTS_25</v>
+      </c>
+      <c r="C409" t="str">
+        <v>10,7798043</v>
+      </c>
+      <c r="D409" t="str">
+        <v>106,6838591</v>
+      </c>
+      <c r="E409" t="str">
+        <v/>
+      </c>
+      <c r="F409" t="str">
+        <v/>
+      </c>
+      <c r="G409" t="str">
+        <v>1</v>
+      </c>
+      <c r="H409" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I409" t="str">
+        <v/>
+      </c>
+      <c r="J409" t="str">
+        <v/>
+      </c>
+      <c r="K409" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L409" t="str">
+        <v/>
+      </c>
+      <c r="M409" t="str">
+        <v/>
+      </c>
+      <c r="N409" t="str">
+        <v>11:29:01 11/6/2026</v>
+      </c>
+      <c r="O409" t="str">
+        <v>VTS_H232VTS_24</v>
+      </c>
+      <c r="P409" t="str">
+        <v/>
+      </c>
+      <c r="Q409" t="str">
+        <v/>
+      </c>
+      <c r="R409" t="str">
+        <v/>
+      </c>
+      <c r="S409" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v/>
+      </c>
+      <c r="B410" t="str">
+        <v>VTS_H232VTS_26</v>
+      </c>
+      <c r="C410" t="str">
+        <v>10,7796366</v>
+      </c>
+      <c r="D410" t="str">
+        <v>106,6837012</v>
+      </c>
+      <c r="E410" t="str">
+        <v/>
+      </c>
+      <c r="F410" t="str">
+        <v/>
+      </c>
+      <c r="G410" t="str">
+        <v>1</v>
+      </c>
+      <c r="H410" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I410" t="str">
+        <v/>
+      </c>
+      <c r="J410" t="str">
+        <v/>
+      </c>
+      <c r="K410" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L410" t="str">
+        <v/>
+      </c>
+      <c r="M410" t="str">
+        <v/>
+      </c>
+      <c r="N410" t="str">
+        <v>16:01:17 10/6/2026</v>
+      </c>
+      <c r="O410" t="str">
+        <v>VTS_H232VTS_25</v>
+      </c>
+      <c r="P410" t="str">
+        <v/>
+      </c>
+      <c r="Q410" t="str">
+        <v/>
+      </c>
+      <c r="R410" t="str">
+        <v/>
+      </c>
+      <c r="S410" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v/>
+      </c>
+      <c r="B411" t="str">
+        <v>VTS_H232VTS_27</v>
+      </c>
+      <c r="C411" t="str">
+        <v>10,7793994</v>
+      </c>
+      <c r="D411" t="str">
+        <v>106,6834532</v>
+      </c>
+      <c r="E411" t="str">
+        <v/>
+      </c>
+      <c r="F411" t="str">
+        <v/>
+      </c>
+      <c r="G411" t="str">
+        <v>1</v>
+      </c>
+      <c r="H411" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I411" t="str">
+        <v/>
+      </c>
+      <c r="J411" t="str">
+        <v/>
+      </c>
+      <c r="K411" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L411" t="str">
+        <v/>
+      </c>
+      <c r="M411" t="str">
+        <v/>
+      </c>
+      <c r="N411" t="str">
+        <v>16:01:12 10/6/2026</v>
+      </c>
+      <c r="O411" t="str">
+        <v>VTS_H232VTS_26</v>
+      </c>
+      <c r="P411" t="str">
+        <v/>
+      </c>
+      <c r="Q411" t="str">
+        <v/>
+      </c>
+      <c r="R411" t="str">
+        <v/>
+      </c>
+      <c r="S411" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v/>
+      </c>
+      <c r="B412" t="str">
+        <v>VTS_H232VTS_28</v>
+      </c>
+      <c r="C412" t="str">
+        <v>10,7791588</v>
+      </c>
+      <c r="D412" t="str">
+        <v>106,6832381</v>
+      </c>
+      <c r="E412" t="str">
+        <v/>
+      </c>
+      <c r="F412" t="str">
+        <v/>
+      </c>
+      <c r="G412" t="str">
+        <v>1</v>
+      </c>
+      <c r="H412" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I412" t="str">
+        <v/>
+      </c>
+      <c r="J412" t="str">
+        <v/>
+      </c>
+      <c r="K412" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L412" t="str">
+        <v/>
+      </c>
+      <c r="M412" t="str">
+        <v/>
+      </c>
+      <c r="N412" t="str">
+        <v>11:28:56 11/6/2026</v>
+      </c>
+      <c r="O412" t="str">
+        <v>VTS_H232VTS_27</v>
+      </c>
+      <c r="P412" t="str">
+        <v/>
+      </c>
+      <c r="Q412" t="str">
+        <v/>
+      </c>
+      <c r="R412" t="str">
+        <v/>
+      </c>
+      <c r="S412" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v/>
+      </c>
+      <c r="B413" t="str">
+        <v>VTS_H232VTS_29</v>
+      </c>
+      <c r="C413" t="str">
+        <v>10,7789368</v>
+      </c>
+      <c r="D413" t="str">
+        <v>106,6830491</v>
+      </c>
+      <c r="E413" t="str">
+        <v/>
+      </c>
+      <c r="F413" t="str">
+        <v/>
+      </c>
+      <c r="G413" t="str">
+        <v>1</v>
+      </c>
+      <c r="H413" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I413" t="str">
+        <v/>
+      </c>
+      <c r="J413" t="str">
+        <v/>
+      </c>
+      <c r="K413" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L413" t="str">
+        <v/>
+      </c>
+      <c r="M413" t="str">
+        <v/>
+      </c>
+      <c r="N413" t="str">
+        <v>11:28:32 11/6/2026</v>
+      </c>
+      <c r="O413" t="str">
+        <v>VTS_H232VTS_28</v>
+      </c>
+      <c r="P413" t="str">
+        <v/>
+      </c>
+      <c r="Q413" t="str">
+        <v/>
+      </c>
+      <c r="R413" t="str">
+        <v/>
+      </c>
+      <c r="S413" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v/>
+      </c>
+      <c r="B414" t="str">
+        <v>VTS_H232VTS_30</v>
+      </c>
+      <c r="C414" t="str">
+        <v>10,7786957</v>
+      </c>
+      <c r="D414" t="str">
+        <v>106,6828311</v>
+      </c>
+      <c r="E414" t="str">
+        <v/>
+      </c>
+      <c r="F414" t="str">
+        <v/>
+      </c>
+      <c r="G414" t="str">
+        <v>1</v>
+      </c>
+      <c r="H414" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I414" t="str">
+        <v/>
+      </c>
+      <c r="J414" t="str">
+        <v/>
+      </c>
+      <c r="K414" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L414" t="str">
+        <v/>
+      </c>
+      <c r="M414" t="str">
+        <v/>
+      </c>
+      <c r="N414" t="str">
+        <v>11:28:25 11/6/2026</v>
+      </c>
+      <c r="O414" t="str">
+        <v>VTS_H232VTS_29</v>
+      </c>
+      <c r="P414" t="str">
+        <v/>
+      </c>
+      <c r="Q414" t="str">
+        <v/>
+      </c>
+      <c r="R414" t="str">
+        <v/>
+      </c>
+      <c r="S414" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v/>
+      </c>
+      <c r="B415" t="str">
+        <v>VTS_H232VTS_31</v>
+      </c>
+      <c r="C415" t="str">
+        <v>10,7784931</v>
+      </c>
+      <c r="D415" t="str">
+        <v>106,6826397</v>
+      </c>
+      <c r="E415" t="str">
+        <v/>
+      </c>
+      <c r="F415" t="str">
+        <v/>
+      </c>
+      <c r="G415" t="str">
+        <v>1</v>
+      </c>
+      <c r="H415" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I415" t="str">
+        <v/>
+      </c>
+      <c r="J415" t="str">
+        <v/>
+      </c>
+      <c r="K415" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L415" t="str">
+        <v/>
+      </c>
+      <c r="M415" t="str">
+        <v/>
+      </c>
+      <c r="N415" t="str">
+        <v>11:28:19 11/6/2026</v>
+      </c>
+      <c r="O415" t="str">
+        <v>VTS_H232VTS_30</v>
+      </c>
+      <c r="P415" t="str">
+        <v/>
+      </c>
+      <c r="Q415" t="str">
+        <v/>
+      </c>
+      <c r="R415" t="str">
+        <v/>
+      </c>
+      <c r="S415" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v/>
+      </c>
+      <c r="B416" t="str">
+        <v>VTS_H232VTS_32</v>
+      </c>
+      <c r="C416" t="str">
+        <v>10,7783584</v>
+      </c>
+      <c r="D416" t="str">
+        <v>106,6824707</v>
+      </c>
+      <c r="E416" t="str">
+        <v/>
+      </c>
+      <c r="F416" t="str">
+        <v/>
+      </c>
+      <c r="G416" t="str">
+        <v>1</v>
+      </c>
+      <c r="H416" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I416" t="str">
+        <v/>
+      </c>
+      <c r="J416" t="str">
+        <v/>
+      </c>
+      <c r="K416" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L416" t="str">
+        <v/>
+      </c>
+      <c r="M416" t="str">
+        <v/>
+      </c>
+      <c r="N416" t="str">
+        <v>11:28:16 11/6/2026</v>
+      </c>
+      <c r="O416" t="str">
+        <v>VTS_H232VTS_31</v>
+      </c>
+      <c r="P416" t="str">
+        <v/>
+      </c>
+      <c r="Q416" t="str">
+        <v/>
+      </c>
+      <c r="R416" t="str">
+        <v/>
+      </c>
+      <c r="S416" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v/>
+      </c>
+      <c r="B417" t="str">
+        <v>VTS_H232VTS_33</v>
+      </c>
+      <c r="C417" t="str">
+        <v>10,7780488</v>
+      </c>
+      <c r="D417" t="str">
+        <v>106,6821726</v>
+      </c>
+      <c r="E417" t="str">
+        <v/>
+      </c>
+      <c r="F417" t="str">
+        <v/>
+      </c>
+      <c r="G417" t="str">
+        <v>1</v>
+      </c>
+      <c r="H417" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I417" t="str">
+        <v/>
+      </c>
+      <c r="J417" t="str">
+        <v/>
+      </c>
+      <c r="K417" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L417" t="str">
+        <v/>
+      </c>
+      <c r="M417" t="str">
+        <v/>
+      </c>
+      <c r="N417" t="str">
+        <v>11:27:59 11/6/2026</v>
+      </c>
+      <c r="O417" t="str">
+        <v>VTS_H232VTS_32</v>
+      </c>
+      <c r="P417" t="str">
+        <v/>
+      </c>
+      <c r="Q417" t="str">
+        <v/>
+      </c>
+      <c r="R417" t="str">
+        <v/>
+      </c>
+      <c r="S417" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v/>
+      </c>
+      <c r="B418" t="str">
+        <v>VTS_H232VTS_34</v>
+      </c>
+      <c r="C418" t="str">
+        <v>10,7779052</v>
+      </c>
+      <c r="D418" t="str">
+        <v>106,6819990</v>
+      </c>
+      <c r="E418" t="str">
+        <v/>
+      </c>
+      <c r="F418" t="str">
+        <v/>
+      </c>
+      <c r="G418" t="str">
+        <v>1</v>
+      </c>
+      <c r="H418" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I418" t="str">
+        <v/>
+      </c>
+      <c r="J418" t="str">
+        <v/>
+      </c>
+      <c r="K418" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L418" t="str">
+        <v/>
+      </c>
+      <c r="M418" t="str">
+        <v/>
+      </c>
+      <c r="N418" t="str">
+        <v>11:27:51 11/6/2026</v>
+      </c>
+      <c r="O418" t="str">
+        <v>VTS_H232VTS_33</v>
+      </c>
+      <c r="P418" t="str">
+        <v/>
+      </c>
+      <c r="Q418" t="str">
+        <v/>
+      </c>
+      <c r="R418" t="str">
+        <v/>
+      </c>
+      <c r="S418" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v/>
+      </c>
+      <c r="B419" t="str">
+        <v>VTS_H23VTS</v>
+      </c>
+      <c r="C419" t="str">
+        <v>10,7818002</v>
+      </c>
+      <c r="D419" t="str">
+        <v>106,6858573</v>
+      </c>
+      <c r="E419" t="str">
+        <v/>
+      </c>
+      <c r="F419" t="str">
+        <v>Admintrator</v>
+      </c>
+      <c r="G419" t="str">
+        <v>6</v>
+      </c>
+      <c r="H419" t="str">
+        <v>VTS_H232VTS</v>
+      </c>
+      <c r="I419" t="str">
+        <v>Tủ chiếu sáng ngầm</v>
+      </c>
+      <c r="J419" t="str">
+        <v/>
+      </c>
+      <c r="K419" t="str">
+        <v>LED</v>
+      </c>
+      <c r="L419" t="str">
+        <v/>
+      </c>
+      <c r="M419" t="str">
+        <v/>
+      </c>
+      <c r="N419" t="str">
+        <v>13:17:54 11/6/2026</v>
+      </c>
+      <c r="O419" t="str">
+        <v>VTS_H232VTS_34</v>
+      </c>
+      <c r="P419" t="str">
+        <v/>
+      </c>
+      <c r="Q419" t="str">
+        <v/>
+      </c>
+      <c r="R419" t="str">
+        <v>Hẻm 232 Võ Thị Sáu</v>
+      </c>
+      <c r="S419" t="str">
+        <v>Phường Xuân Hòa</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S372"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S419"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Đồng bộ dữ liệu khảo sát 2026-06-18
</commit_message>
<xml_diff>
--- a/data/khaosat.xlsx
+++ b/data/khaosat.xlsx
@@ -12761,10 +12761,10 @@
         <v>Bình Dương 952</v>
       </c>
       <c r="C175" t="str">
-        <v>11,1947439</v>
+        <v>11,1951511</v>
       </c>
       <c r="D175" t="str">
-        <v>106,6294094</v>
+        <v>106,6295336</v>
       </c>
       <c r="E175" t="str">
         <v>Phường Bến Cát, Thành phố Hồ Chí Minh, Việt Nam</v>
@@ -12794,7 +12794,7 @@
         <v/>
       </c>
       <c r="N175" t="str">
-        <v/>
+        <v>08:32:23 18/6/2026</v>
       </c>
       <c r="O175" t="str">
         <v/>
@@ -12812,16 +12812,16 @@
         <v>Phường Bến Cát</v>
       </c>
       <c r="T175" t="str">
-        <v/>
+        <v>677921</v>
       </c>
       <c r="U175" t="str">
-        <v/>
+        <v>1238049</v>
       </c>
       <c r="V175" t="str">
         <v/>
       </c>
       <c r="W175" t="str">
-        <v/>
+        <v>noi</v>
       </c>
     </row>
     <row r="176">
@@ -15459,10 +15459,10 @@
         <v>CS Bình Dương 2062</v>
       </c>
       <c r="C213" t="str">
-        <v>11,1883853</v>
+        <v>11,1878547</v>
       </c>
       <c r="D213" t="str">
-        <v>106,6310941</v>
+        <v>106,6310064</v>
       </c>
       <c r="E213" t="str">
         <v>Phường Bến Cát, Thành phố Hồ Chí Minh, Việt Nam</v>
@@ -15492,7 +15492,7 @@
         <v/>
       </c>
       <c r="N213" t="str">
-        <v/>
+        <v>08:50:11 18/6/2026</v>
       </c>
       <c r="O213" t="str">
         <v/>
@@ -15510,16 +15510,16 @@
         <v>Phường Bến Cát</v>
       </c>
       <c r="T213" t="str">
-        <v/>
+        <v>678086</v>
       </c>
       <c r="U213" t="str">
-        <v/>
+        <v>1237243</v>
       </c>
       <c r="V213" t="str">
         <v/>
       </c>
       <c r="W213" t="str">
-        <v/>
+        <v>noi</v>
       </c>
     </row>
     <row r="214">

</xml_diff>

<commit_message>
Đồng bộ dữ liệu khảo sát 2026-07-06
</commit_message>
<xml_diff>
--- a/data/khaosat.xlsx
+++ b/data/khaosat.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z425"/>
+  <dimension ref="A1:Z402"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13696,16 +13696,16 @@
         <v>Mỹ Thạnh, Bến Cát, Phường Bến Cát, Thành phố Hồ Chí Minh, 75911, Việt Nam</v>
       </c>
       <c r="F167" t="str">
-        <v>Nguyễn Gia Lâm</v>
+        <v>Admintrator</v>
       </c>
       <c r="G167" t="str">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H167" t="str">
         <v>102.166.000</v>
       </c>
       <c r="I167" t="str">
-        <v/>
+        <v>Tủ chiếu sáng nổi</v>
       </c>
       <c r="J167" t="str">
         <v/>
@@ -13720,13 +13720,13 @@
         <v/>
       </c>
       <c r="N167" t="str">
-        <v/>
+        <v>11:54:29 2/7/2026</v>
       </c>
       <c r="O167" t="str">
-        <v/>
+        <v>CS Bình Dương 2267</v>
       </c>
       <c r="P167" t="str">
-        <v/>
+        <v>24302</v>
       </c>
       <c r="Q167" t="str">
         <v/>
@@ -13747,7 +13747,7 @@
         <v/>
       </c>
       <c r="W167" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X167" t="str">
         <v/>
@@ -31121,73 +31121,73 @@
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v/>
+        <v>16316_1</v>
       </c>
       <c r="B385" t="str">
-        <v>DBP_DBP6_1</v>
+        <v>ADV_ADV_3_1</v>
       </c>
       <c r="C385" t="str">
-        <v>10,7812877</v>
+        <v>10,7602555</v>
       </c>
       <c r="D385" t="str">
-        <v>106,6885735</v>
+        <v>106,6807705</v>
       </c>
       <c r="E385" t="str">
         <v/>
       </c>
       <c r="F385" t="str">
-        <v>Admintrator</v>
+        <v/>
       </c>
       <c r="G385" t="str">
+        <v>3</v>
+      </c>
+      <c r="H385" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I385" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J385" t="str">
+        <v/>
+      </c>
+      <c r="K385" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L385" t="str">
+        <v>250</v>
+      </c>
+      <c r="M385" t="str">
+        <v/>
+      </c>
+      <c r="N385" t="str">
+        <v>13:31:35 6/7/2026</v>
+      </c>
+      <c r="O385" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="P385" t="str">
+        <v/>
+      </c>
+      <c r="Q385" t="str">
+        <v/>
+      </c>
+      <c r="R385" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S385" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T385" t="str">
+        <v>683785</v>
+      </c>
+      <c r="U385" t="str">
+        <v>1189974</v>
+      </c>
+      <c r="V385" t="str">
         <v>1</v>
       </c>
-      <c r="H385" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I385" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J385" t="str">
-        <v/>
-      </c>
-      <c r="K385" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L385" t="str">
-        <v>100</v>
-      </c>
-      <c r="M385" t="str">
-        <v>https://raw.githubusercontent.com/neo-era/lighting-survey/main/images/vts-h232vts-1-2026-06-12T06-24-03Z.png</v>
-      </c>
-      <c r="N385" t="str">
-        <v>10:57:51 15/6/2026</v>
-      </c>
-      <c r="O385" t="str">
-        <v>VTS_H232VTS_1</v>
-      </c>
-      <c r="P385" t="str">
-        <v>0</v>
-      </c>
-      <c r="Q385" t="str">
-        <v/>
-      </c>
-      <c r="R385" t="str">
-        <v>Đường Võ Thị Sáu</v>
-      </c>
-      <c r="S385" t="str">
-        <v/>
-      </c>
-      <c r="T385" t="str">
-        <v>684615</v>
-      </c>
-      <c r="U385" t="str">
-        <v>1192657</v>
-      </c>
-      <c r="V385" t="str">
-        <v>4</v>
-      </c>
       <c r="W385" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X385" t="str">
         <v/>
@@ -31201,73 +31201,73 @@
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v/>
+        <v>16316_2</v>
       </c>
       <c r="B386" t="str">
-        <v>DBP_DBP6_2</v>
+        <v>ADV_ADV_3_2</v>
       </c>
       <c r="C386" t="str">
-        <v>10,7815442</v>
+        <v>10,7601721</v>
       </c>
       <c r="D386" t="str">
-        <v>106,6888539</v>
+        <v>106,6805621</v>
       </c>
       <c r="E386" t="str">
         <v/>
       </c>
       <c r="F386" t="str">
-        <v>Admintrator</v>
+        <v/>
       </c>
       <c r="G386" t="str">
+        <v>3</v>
+      </c>
+      <c r="H386" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I386" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J386" t="str">
+        <v/>
+      </c>
+      <c r="K386" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L386" t="str">
+        <v>250</v>
+      </c>
+      <c r="M386" t="str">
+        <v/>
+      </c>
+      <c r="N386" t="str">
+        <v>16:09:33 6/7/2026</v>
+      </c>
+      <c r="O386" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="P386" t="str">
+        <v/>
+      </c>
+      <c r="Q386" t="str">
+        <v/>
+      </c>
+      <c r="R386" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S386" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T386" t="str">
+        <v>683763</v>
+      </c>
+      <c r="U386" t="str">
+        <v>1189965</v>
+      </c>
+      <c r="V386" t="str">
         <v>1</v>
       </c>
-      <c r="H386" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I386" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J386" t="str">
-        <v/>
-      </c>
-      <c r="K386" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L386" t="str">
-        <v>120</v>
-      </c>
-      <c r="M386" t="str">
-        <v/>
-      </c>
-      <c r="N386" t="str">
-        <v>18:24:05 15/6/2026</v>
-      </c>
-      <c r="O386" t="str">
-        <v>VTS_H232VTS_1</v>
-      </c>
-      <c r="P386" t="str">
-        <v>42</v>
-      </c>
-      <c r="Q386" t="str">
-        <v/>
-      </c>
-      <c r="R386" t="str">
-        <v/>
-      </c>
-      <c r="S386" t="str">
-        <v/>
-      </c>
-      <c r="T386" t="str">
-        <v>684585</v>
-      </c>
-      <c r="U386" t="str">
-        <v>1192629</v>
-      </c>
-      <c r="V386" t="str">
-        <v>2</v>
-      </c>
       <c r="W386" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X386" t="str">
         <v/>
@@ -31281,16 +31281,16 @@
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v/>
+        <v>16316_3</v>
       </c>
       <c r="B387" t="str">
-        <v>DBP_DBP6_3</v>
+        <v>ADV_ADV_3_3</v>
       </c>
       <c r="C387" t="str">
-        <v>10,7817618</v>
+        <v>10,7600177</v>
       </c>
       <c r="D387" t="str">
-        <v>106,6890827</v>
+        <v>106,6801760</v>
       </c>
       <c r="E387" t="str">
         <v/>
@@ -31299,55 +31299,55 @@
         <v/>
       </c>
       <c r="G387" t="str">
+        <v>3</v>
+      </c>
+      <c r="H387" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I387" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J387" t="str">
+        <v/>
+      </c>
+      <c r="K387" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L387" t="str">
+        <v>250</v>
+      </c>
+      <c r="M387" t="str">
+        <v/>
+      </c>
+      <c r="N387" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O387" t="str">
+        <v>ADV_ADV_3_2</v>
+      </c>
+      <c r="P387" t="str">
+        <v/>
+      </c>
+      <c r="Q387" t="str">
+        <v/>
+      </c>
+      <c r="R387" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S387" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T387" t="str">
+        <v>683720</v>
+      </c>
+      <c r="U387" t="str">
+        <v>1189948</v>
+      </c>
+      <c r="V387" t="str">
         <v>1</v>
       </c>
-      <c r="H387" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I387" t="str">
-        <v/>
-      </c>
-      <c r="J387" t="str">
-        <v/>
-      </c>
-      <c r="K387" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L387" t="str">
-        <v/>
-      </c>
-      <c r="M387" t="str">
-        <v/>
-      </c>
-      <c r="N387" t="str">
-        <v>11:32:31 11/6/2026</v>
-      </c>
-      <c r="O387" t="str">
-        <v>VTS_H232VTS_2</v>
-      </c>
-      <c r="P387" t="str">
-        <v/>
-      </c>
-      <c r="Q387" t="str">
-        <v/>
-      </c>
-      <c r="R387" t="str">
-        <v/>
-      </c>
-      <c r="S387" t="str">
-        <v/>
-      </c>
-      <c r="T387" t="str">
-        <v>684566</v>
-      </c>
-      <c r="U387" t="str">
-        <v>1192608</v>
-      </c>
-      <c r="V387" t="str">
-        <v/>
-      </c>
       <c r="W387" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X387" t="str">
         <v/>
@@ -31361,16 +31361,16 @@
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v/>
+        <v>16316_4</v>
       </c>
       <c r="B388" t="str">
-        <v>DBP_DBP6_4</v>
+        <v>ADV_ADV_3_4</v>
       </c>
       <c r="C388" t="str">
-        <v>10,7819207</v>
+        <v>10,7599300</v>
       </c>
       <c r="D388" t="str">
-        <v>106,6892401</v>
+        <v>106,6799568</v>
       </c>
       <c r="E388" t="str">
         <v/>
@@ -31379,55 +31379,55 @@
         <v/>
       </c>
       <c r="G388" t="str">
+        <v>3</v>
+      </c>
+      <c r="H388" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I388" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J388" t="str">
+        <v/>
+      </c>
+      <c r="K388" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L388" t="str">
+        <v>250</v>
+      </c>
+      <c r="M388" t="str">
+        <v/>
+      </c>
+      <c r="N388" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O388" t="str">
+        <v>ADV_ADV_3_3</v>
+      </c>
+      <c r="P388" t="str">
+        <v/>
+      </c>
+      <c r="Q388" t="str">
+        <v/>
+      </c>
+      <c r="R388" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S388" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T388" t="str">
+        <v>683696</v>
+      </c>
+      <c r="U388" t="str">
+        <v>1189938</v>
+      </c>
+      <c r="V388" t="str">
         <v>1</v>
       </c>
-      <c r="H388" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I388" t="str">
-        <v/>
-      </c>
-      <c r="J388" t="str">
-        <v/>
-      </c>
-      <c r="K388" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L388" t="str">
-        <v/>
-      </c>
-      <c r="M388" t="str">
-        <v/>
-      </c>
-      <c r="N388" t="str">
-        <v>11:32:28 11/6/2026</v>
-      </c>
-      <c r="O388" t="str">
-        <v>VTS_H232VTS_3</v>
-      </c>
-      <c r="P388" t="str">
-        <v/>
-      </c>
-      <c r="Q388" t="str">
-        <v/>
-      </c>
-      <c r="R388" t="str">
-        <v/>
-      </c>
-      <c r="S388" t="str">
-        <v/>
-      </c>
-      <c r="T388" t="str">
-        <v>684540</v>
-      </c>
-      <c r="U388" t="str">
-        <v>1192582</v>
-      </c>
-      <c r="V388" t="str">
-        <v/>
-      </c>
       <c r="W388" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X388" t="str">
         <v/>
@@ -31441,16 +31441,16 @@
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v/>
+        <v>16316_5</v>
       </c>
       <c r="B389" t="str">
-        <v>DBP_DBP6_5</v>
+        <v>ADV_ADV_3_5</v>
       </c>
       <c r="C389" t="str">
-        <v>10,7821553</v>
+        <v>10,7598328</v>
       </c>
       <c r="D389" t="str">
-        <v>106,6894691</v>
+        <v>106,6797138</v>
       </c>
       <c r="E389" t="str">
         <v/>
@@ -31459,55 +31459,55 @@
         <v/>
       </c>
       <c r="G389" t="str">
+        <v>3</v>
+      </c>
+      <c r="H389" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I389" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J389" t="str">
+        <v/>
+      </c>
+      <c r="K389" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L389" t="str">
+        <v>250</v>
+      </c>
+      <c r="M389" t="str">
+        <v/>
+      </c>
+      <c r="N389" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O389" t="str">
+        <v>ADV_ADV_3_4</v>
+      </c>
+      <c r="P389" t="str">
+        <v/>
+      </c>
+      <c r="Q389" t="str">
+        <v/>
+      </c>
+      <c r="R389" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S389" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T389" t="str">
+        <v>683670</v>
+      </c>
+      <c r="U389" t="str">
+        <v>1189927</v>
+      </c>
+      <c r="V389" t="str">
         <v>1</v>
       </c>
-      <c r="H389" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I389" t="str">
-        <v/>
-      </c>
-      <c r="J389" t="str">
-        <v/>
-      </c>
-      <c r="K389" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L389" t="str">
-        <v/>
-      </c>
-      <c r="M389" t="str">
-        <v/>
-      </c>
-      <c r="N389" t="str">
-        <v>11:30:18 11/6/2026</v>
-      </c>
-      <c r="O389" t="str">
-        <v>VTS_H232VTS_4</v>
-      </c>
-      <c r="P389" t="str">
-        <v/>
-      </c>
-      <c r="Q389" t="str">
-        <v/>
-      </c>
-      <c r="R389" t="str">
-        <v/>
-      </c>
-      <c r="S389" t="str">
-        <v/>
-      </c>
-      <c r="T389" t="str">
-        <v>684519</v>
-      </c>
-      <c r="U389" t="str">
-        <v>1192554</v>
-      </c>
-      <c r="V389" t="str">
-        <v/>
-      </c>
       <c r="W389" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X389" t="str">
         <v/>
@@ -31521,16 +31521,16 @@
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v/>
+        <v>16316_6</v>
       </c>
       <c r="B390" t="str">
-        <v>DBP_DBP6_6</v>
+        <v>ADV_ADV_3_6</v>
       </c>
       <c r="C390" t="str">
-        <v>10,7824765</v>
+        <v>10,7597156</v>
       </c>
       <c r="D390" t="str">
-        <v>106,6898277</v>
+        <v>106,6794209</v>
       </c>
       <c r="E390" t="str">
         <v/>
@@ -31539,55 +31539,55 @@
         <v/>
       </c>
       <c r="G390" t="str">
+        <v>3</v>
+      </c>
+      <c r="H390" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I390" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J390" t="str">
+        <v/>
+      </c>
+      <c r="K390" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L390" t="str">
+        <v>250</v>
+      </c>
+      <c r="M390" t="str">
+        <v/>
+      </c>
+      <c r="N390" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O390" t="str">
+        <v>ADV_ADV_3_5</v>
+      </c>
+      <c r="P390" t="str">
+        <v/>
+      </c>
+      <c r="Q390" t="str">
+        <v/>
+      </c>
+      <c r="R390" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S390" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T390" t="str">
+        <v>683638</v>
+      </c>
+      <c r="U390" t="str">
+        <v>1189914</v>
+      </c>
+      <c r="V390" t="str">
         <v>1</v>
       </c>
-      <c r="H390" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I390" t="str">
-        <v/>
-      </c>
-      <c r="J390" t="str">
-        <v/>
-      </c>
-      <c r="K390" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L390" t="str">
-        <v/>
-      </c>
-      <c r="M390" t="str">
-        <v/>
-      </c>
-      <c r="N390" t="str">
-        <v>11:32:06 11/6/2026</v>
-      </c>
-      <c r="O390" t="str">
-        <v>VTS_H232VTS_5</v>
-      </c>
-      <c r="P390" t="str">
-        <v/>
-      </c>
-      <c r="Q390" t="str">
-        <v/>
-      </c>
-      <c r="R390" t="str">
-        <v/>
-      </c>
-      <c r="S390" t="str">
-        <v/>
-      </c>
-      <c r="T390" t="str">
-        <v>684479</v>
-      </c>
-      <c r="U390" t="str">
-        <v>1192516</v>
-      </c>
-      <c r="V390" t="str">
-        <v/>
-      </c>
       <c r="W390" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X390" t="str">
         <v/>
@@ -31601,16 +31601,16 @@
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v/>
+        <v>16316_7</v>
       </c>
       <c r="B391" t="str">
-        <v>DBP_DBP6_7</v>
+        <v>ADV_ADV_3_7</v>
       </c>
       <c r="C391" t="str">
-        <v>10,7826892</v>
+        <v>10,7595922</v>
       </c>
       <c r="D391" t="str">
-        <v>106,6900193</v>
+        <v>106,6791126</v>
       </c>
       <c r="E391" t="str">
         <v/>
@@ -31619,55 +31619,55 @@
         <v/>
       </c>
       <c r="G391" t="str">
+        <v>3</v>
+      </c>
+      <c r="H391" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I391" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J391" t="str">
+        <v/>
+      </c>
+      <c r="K391" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L391" t="str">
+        <v>250</v>
+      </c>
+      <c r="M391" t="str">
+        <v/>
+      </c>
+      <c r="N391" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O391" t="str">
+        <v>ADV_ADV_3_6</v>
+      </c>
+      <c r="P391" t="str">
+        <v/>
+      </c>
+      <c r="Q391" t="str">
+        <v/>
+      </c>
+      <c r="R391" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S391" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T391" t="str">
+        <v>683604</v>
+      </c>
+      <c r="U391" t="str">
+        <v>1189900</v>
+      </c>
+      <c r="V391" t="str">
         <v>1</v>
       </c>
-      <c r="H391" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I391" t="str">
-        <v/>
-      </c>
-      <c r="J391" t="str">
-        <v/>
-      </c>
-      <c r="K391" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L391" t="str">
-        <v/>
-      </c>
-      <c r="M391" t="str">
-        <v/>
-      </c>
-      <c r="N391" t="str">
-        <v>11:32:02 11/6/2026</v>
-      </c>
-      <c r="O391" t="str">
-        <v>VTS_H232VTS_6</v>
-      </c>
-      <c r="P391" t="str">
-        <v/>
-      </c>
-      <c r="Q391" t="str">
-        <v/>
-      </c>
-      <c r="R391" t="str">
-        <v/>
-      </c>
-      <c r="S391" t="str">
-        <v/>
-      </c>
-      <c r="T391" t="str">
-        <v>684495</v>
-      </c>
-      <c r="U391" t="str">
-        <v>1192532</v>
-      </c>
-      <c r="V391" t="str">
-        <v/>
-      </c>
       <c r="W391" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X391" t="str">
         <v/>
@@ -31681,16 +31681,16 @@
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v/>
+        <v>16316_8</v>
       </c>
       <c r="B392" t="str">
-        <v>DBP_DBP6_8</v>
+        <v>ADV_ADV_3_8</v>
       </c>
       <c r="C392" t="str">
-        <v>10,7828849</v>
+        <v>10,7594752</v>
       </c>
       <c r="D392" t="str">
-        <v>106,6902408</v>
+        <v>106,6788201</v>
       </c>
       <c r="E392" t="str">
         <v/>
@@ -31699,55 +31699,55 @@
         <v/>
       </c>
       <c r="G392" t="str">
+        <v>3</v>
+      </c>
+      <c r="H392" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I392" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J392" t="str">
+        <v/>
+      </c>
+      <c r="K392" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L392" t="str">
+        <v>250</v>
+      </c>
+      <c r="M392" t="str">
+        <v/>
+      </c>
+      <c r="N392" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O392" t="str">
+        <v>ADV_ADV_3_7</v>
+      </c>
+      <c r="P392" t="str">
+        <v/>
+      </c>
+      <c r="Q392" t="str">
+        <v/>
+      </c>
+      <c r="R392" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S392" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T392" t="str">
+        <v>683572</v>
+      </c>
+      <c r="U392" t="str">
+        <v>1189887</v>
+      </c>
+      <c r="V392" t="str">
         <v>1</v>
       </c>
-      <c r="H392" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I392" t="str">
-        <v/>
-      </c>
-      <c r="J392" t="str">
-        <v/>
-      </c>
-      <c r="K392" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L392" t="str">
-        <v/>
-      </c>
-      <c r="M392" t="str">
-        <v/>
-      </c>
-      <c r="N392" t="str">
-        <v>11:32:15 11/6/2026</v>
-      </c>
-      <c r="O392" t="str">
-        <v>VTS_H232VTS_7</v>
-      </c>
-      <c r="P392" t="str">
-        <v/>
-      </c>
-      <c r="Q392" t="str">
-        <v/>
-      </c>
-      <c r="R392" t="str">
-        <v/>
-      </c>
-      <c r="S392" t="str">
-        <v/>
-      </c>
-      <c r="T392" t="str">
-        <v>684463</v>
-      </c>
-      <c r="U392" t="str">
-        <v>1192499</v>
-      </c>
-      <c r="V392" t="str">
-        <v/>
-      </c>
       <c r="W392" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X392" t="str">
         <v/>
@@ -31761,16 +31761,16 @@
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v/>
+        <v>16316_9</v>
       </c>
       <c r="B393" t="str">
-        <v>DBP_DBP6_9</v>
+        <v>ADV_ADV_3_9</v>
       </c>
       <c r="C393" t="str">
-        <v>10,7831094</v>
+        <v>10,7593637</v>
       </c>
       <c r="D393" t="str">
-        <v>106,6904690</v>
+        <v>106,6785415</v>
       </c>
       <c r="E393" t="str">
         <v/>
@@ -31779,55 +31779,55 @@
         <v/>
       </c>
       <c r="G393" t="str">
+        <v>3</v>
+      </c>
+      <c r="H393" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I393" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J393" t="str">
+        <v/>
+      </c>
+      <c r="K393" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L393" t="str">
+        <v>250</v>
+      </c>
+      <c r="M393" t="str">
+        <v/>
+      </c>
+      <c r="N393" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O393" t="str">
+        <v>ADV_ADV_3_8</v>
+      </c>
+      <c r="P393" t="str">
+        <v/>
+      </c>
+      <c r="Q393" t="str">
+        <v/>
+      </c>
+      <c r="R393" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S393" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T393" t="str">
+        <v>683542</v>
+      </c>
+      <c r="U393" t="str">
+        <v>1189874</v>
+      </c>
+      <c r="V393" t="str">
         <v>1</v>
       </c>
-      <c r="H393" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I393" t="str">
-        <v/>
-      </c>
-      <c r="J393" t="str">
-        <v/>
-      </c>
-      <c r="K393" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L393" t="str">
-        <v/>
-      </c>
-      <c r="M393" t="str">
-        <v/>
-      </c>
-      <c r="N393" t="str">
-        <v>15:59:09 12/6/2026</v>
-      </c>
-      <c r="O393" t="str">
-        <v>VTS_H232VTS_8</v>
-      </c>
-      <c r="P393" t="str">
-        <v/>
-      </c>
-      <c r="Q393" t="str">
-        <v/>
-      </c>
-      <c r="R393" t="str">
-        <v/>
-      </c>
-      <c r="S393" t="str">
-        <v/>
-      </c>
-      <c r="T393" t="str">
-        <v>684441</v>
-      </c>
-      <c r="U393" t="str">
-        <v>1192476</v>
-      </c>
-      <c r="V393" t="str">
-        <v/>
-      </c>
       <c r="W393" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X393" t="str">
         <v/>
@@ -31841,16 +31841,16 @@
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v/>
+        <v>16316_10</v>
       </c>
       <c r="B394" t="str">
-        <v>DBP_DBP6_10</v>
+        <v>ADV_ADV_3_10</v>
       </c>
       <c r="C394" t="str">
-        <v>10,7833257</v>
+        <v>10,7592472</v>
       </c>
       <c r="D394" t="str">
-        <v>106,6906826</v>
+        <v>106,6782502</v>
       </c>
       <c r="E394" t="str">
         <v/>
@@ -31859,55 +31859,55 @@
         <v/>
       </c>
       <c r="G394" t="str">
+        <v>3</v>
+      </c>
+      <c r="H394" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I394" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J394" t="str">
+        <v/>
+      </c>
+      <c r="K394" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L394" t="str">
+        <v>250</v>
+      </c>
+      <c r="M394" t="str">
+        <v/>
+      </c>
+      <c r="N394" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O394" t="str">
+        <v>ADV_ADV_3_9</v>
+      </c>
+      <c r="P394" t="str">
+        <v/>
+      </c>
+      <c r="Q394" t="str">
+        <v/>
+      </c>
+      <c r="R394" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S394" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T394" t="str">
+        <v>683510</v>
+      </c>
+      <c r="U394" t="str">
+        <v>1189861</v>
+      </c>
+      <c r="V394" t="str">
         <v>1</v>
       </c>
-      <c r="H394" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I394" t="str">
-        <v/>
-      </c>
-      <c r="J394" t="str">
-        <v/>
-      </c>
-      <c r="K394" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L394" t="str">
-        <v/>
-      </c>
-      <c r="M394" t="str">
-        <v/>
-      </c>
-      <c r="N394" t="str">
-        <v>15:59:04 12/6/2026</v>
-      </c>
-      <c r="O394" t="str">
-        <v>VTS_H232VTS_9</v>
-      </c>
-      <c r="P394" t="str">
-        <v/>
-      </c>
-      <c r="Q394" t="str">
-        <v/>
-      </c>
-      <c r="R394" t="str">
-        <v/>
-      </c>
-      <c r="S394" t="str">
-        <v/>
-      </c>
-      <c r="T394" t="str">
-        <v>684421</v>
-      </c>
-      <c r="U394" t="str">
-        <v>1192458</v>
-      </c>
-      <c r="V394" t="str">
-        <v/>
-      </c>
       <c r="W394" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X394" t="str">
         <v/>
@@ -31921,16 +31921,16 @@
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v/>
+        <v>16316_11</v>
       </c>
       <c r="B395" t="str">
-        <v>DBP_DBP6_11</v>
+        <v>ADV_ADV_3_11</v>
       </c>
       <c r="C395" t="str">
-        <v>10,7835701</v>
+        <v>10,7591425</v>
       </c>
       <c r="D395" t="str">
-        <v>106,6909459</v>
+        <v>106,6779886</v>
       </c>
       <c r="E395" t="str">
         <v/>
@@ -31939,55 +31939,55 @@
         <v/>
       </c>
       <c r="G395" t="str">
+        <v>3</v>
+      </c>
+      <c r="H395" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I395" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J395" t="str">
+        <v/>
+      </c>
+      <c r="K395" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L395" t="str">
+        <v>250</v>
+      </c>
+      <c r="M395" t="str">
+        <v/>
+      </c>
+      <c r="N395" t="str">
+        <v>16:09:49 6/7/2026</v>
+      </c>
+      <c r="O395" t="str">
+        <v>ADV_ADV_3_10</v>
+      </c>
+      <c r="P395" t="str">
+        <v/>
+      </c>
+      <c r="Q395" t="str">
+        <v/>
+      </c>
+      <c r="R395" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S395" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T395" t="str">
+        <v>683482</v>
+      </c>
+      <c r="U395" t="str">
+        <v>1189850</v>
+      </c>
+      <c r="V395" t="str">
         <v>1</v>
       </c>
-      <c r="H395" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I395" t="str">
-        <v/>
-      </c>
-      <c r="J395" t="str">
-        <v/>
-      </c>
-      <c r="K395" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L395" t="str">
-        <v/>
-      </c>
-      <c r="M395" t="str">
-        <v/>
-      </c>
-      <c r="N395" t="str">
-        <v>15:59:06 12/6/2026</v>
-      </c>
-      <c r="O395" t="str">
-        <v>VTS_H232VTS_10</v>
-      </c>
-      <c r="P395" t="str">
-        <v/>
-      </c>
-      <c r="Q395" t="str">
-        <v/>
-      </c>
-      <c r="R395" t="str">
-        <v/>
-      </c>
-      <c r="S395" t="str">
-        <v/>
-      </c>
-      <c r="T395" t="str">
-        <v>684406</v>
-      </c>
-      <c r="U395" t="str">
-        <v>1192442</v>
-      </c>
-      <c r="V395" t="str">
-        <v/>
-      </c>
       <c r="W395" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X395" t="str">
         <v/>
@@ -32001,16 +32001,16 @@
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v/>
+        <v>16316_12</v>
       </c>
       <c r="B396" t="str">
-        <v>DBP_DBP6_12</v>
+        <v>ADV_ADV_3_12</v>
       </c>
       <c r="C396" t="str">
-        <v>10,7837848</v>
+        <v>10,7590408</v>
       </c>
       <c r="D396" t="str">
-        <v>106,6911829</v>
+        <v>106,6777343</v>
       </c>
       <c r="E396" t="str">
         <v/>
@@ -32019,55 +32019,55 @@
         <v/>
       </c>
       <c r="G396" t="str">
+        <v>3</v>
+      </c>
+      <c r="H396" t="str">
+        <v>An Dương Vương - 3</v>
+      </c>
+      <c r="I396" t="str">
+        <v>Trụ bê tông đơn chiếu sáng quản lý</v>
+      </c>
+      <c r="J396" t="str">
+        <v/>
+      </c>
+      <c r="K396" t="str">
+        <v>HPS</v>
+      </c>
+      <c r="L396" t="str">
+        <v>250</v>
+      </c>
+      <c r="M396" t="str">
+        <v/>
+      </c>
+      <c r="N396" t="str">
+        <v>13:31:52 6/7/2026</v>
+      </c>
+      <c r="O396" t="str">
+        <v>ADV_ADV_3_11</v>
+      </c>
+      <c r="P396" t="str">
+        <v/>
+      </c>
+      <c r="Q396" t="str">
+        <v/>
+      </c>
+      <c r="R396" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S396" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T396" t="str">
+        <v>683454</v>
+      </c>
+      <c r="U396" t="str">
+        <v>1189838</v>
+      </c>
+      <c r="V396" t="str">
         <v>1</v>
       </c>
-      <c r="H396" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I396" t="str">
-        <v/>
-      </c>
-      <c r="J396" t="str">
-        <v/>
-      </c>
-      <c r="K396" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L396" t="str">
-        <v/>
-      </c>
-      <c r="M396" t="str">
-        <v/>
-      </c>
-      <c r="N396" t="str">
-        <v>11:15:15 11/6/2026</v>
-      </c>
-      <c r="O396" t="str">
-        <v>VTS_H232VTS_11</v>
-      </c>
-      <c r="P396" t="str">
-        <v/>
-      </c>
-      <c r="Q396" t="str">
-        <v/>
-      </c>
-      <c r="R396" t="str">
-        <v/>
-      </c>
-      <c r="S396" t="str">
-        <v/>
-      </c>
-      <c r="T396" t="str">
-        <v>684389</v>
-      </c>
-      <c r="U396" t="str">
-        <v>1192425</v>
-      </c>
-      <c r="V396" t="str">
-        <v/>
-      </c>
       <c r="W396" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X396" t="str">
         <v/>
@@ -32081,16 +32081,16 @@
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v/>
+        <v>41702_1</v>
       </c>
       <c r="B397" t="str">
-        <v>DBP_DBP6_13</v>
+        <v>H338.ADV_ADV_3_1</v>
       </c>
       <c r="C397" t="str">
-        <v>10,7840059</v>
+        <v>10,7597628</v>
       </c>
       <c r="D397" t="str">
-        <v>106,6914126</v>
+        <v>106,6790968</v>
       </c>
       <c r="E397" t="str">
         <v/>
@@ -32099,13 +32099,13 @@
         <v/>
       </c>
       <c r="G397" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H397" t="str">
-        <v>VTS_H232VTS</v>
+        <v>An Dương Vương - 3</v>
       </c>
       <c r="I397" t="str">
-        <v/>
+        <v>Trụ bê tông đơn điện lực quản lý</v>
       </c>
       <c r="J397" t="str">
         <v/>
@@ -32114,40 +32114,40 @@
         <v>LED</v>
       </c>
       <c r="L397" t="str">
-        <v/>
+        <v>40</v>
       </c>
       <c r="M397" t="str">
         <v/>
       </c>
       <c r="N397" t="str">
-        <v>11:15:18 11/6/2026</v>
+        <v>13:32:04 6/7/2026</v>
       </c>
       <c r="O397" t="str">
-        <v>VTS_H232VTS_12</v>
+        <v>ADV_ADV_3_7</v>
       </c>
       <c r="P397" t="str">
-        <v/>
+        <v>37</v>
       </c>
       <c r="Q397" t="str">
         <v/>
       </c>
       <c r="R397" t="str">
-        <v/>
+        <v>Hẻm 338 An Dương Vương</v>
       </c>
       <c r="S397" t="str">
-        <v/>
+        <v>Phường 4</v>
       </c>
       <c r="T397" t="str">
-        <v>684367</v>
+        <v>683603</v>
       </c>
       <c r="U397" t="str">
-        <v>1192402</v>
+        <v>1189919</v>
       </c>
       <c r="V397" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W397" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X397" t="str">
         <v/>
@@ -32161,16 +32161,16 @@
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v/>
+        <v>41702_2</v>
       </c>
       <c r="B398" t="str">
-        <v>DBP_DBP6_14</v>
+        <v>H338.ADV_ADV_3_2</v>
       </c>
       <c r="C398" t="str">
-        <v>10,7842401</v>
+        <v>10,7599971</v>
       </c>
       <c r="D398" t="str">
-        <v>106,6916172</v>
+        <v>106,6790225</v>
       </c>
       <c r="E398" t="str">
         <v/>
@@ -32179,13 +32179,13 @@
         <v/>
       </c>
       <c r="G398" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H398" t="str">
-        <v>VTS_H232VTS</v>
+        <v>An Dương Vương - 3</v>
       </c>
       <c r="I398" t="str">
-        <v/>
+        <v>Trụ bê tông đơn điện lực quản lý</v>
       </c>
       <c r="J398" t="str">
         <v/>
@@ -32194,16 +32194,16 @@
         <v>LED</v>
       </c>
       <c r="L398" t="str">
-        <v/>
+        <v>40</v>
       </c>
       <c r="M398" t="str">
         <v/>
       </c>
       <c r="N398" t="str">
-        <v>16:36:33 15/6/2026</v>
+        <v>16:09:49 6/7/2026</v>
       </c>
       <c r="O398" t="str">
-        <v>VTS_H232VTS_13</v>
+        <v>H338.ADV_ADV_3_1</v>
       </c>
       <c r="P398" t="str">
         <v/>
@@ -32212,22 +32212,22 @@
         <v/>
       </c>
       <c r="R398" t="str">
-        <v/>
+        <v>Hẻm 338 An Dương Vương</v>
       </c>
       <c r="S398" t="str">
-        <v/>
+        <v>Phường 4</v>
       </c>
       <c r="T398" t="str">
-        <v>684337</v>
+        <v>683594</v>
       </c>
       <c r="U398" t="str">
-        <v>1192376</v>
+        <v>1189945</v>
       </c>
       <c r="V398" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W398" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X398" t="str">
         <v/>
@@ -32241,31 +32241,31 @@
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v/>
+        <v>41702_3</v>
       </c>
       <c r="B399" t="str">
-        <v/>
+        <v>H338.ADV_ADV_3_3</v>
       </c>
       <c r="C399" t="str">
-        <v/>
+        <v>10,7602942</v>
       </c>
       <c r="D399" t="str">
-        <v/>
+        <v>106,6789283</v>
       </c>
       <c r="E399" t="str">
         <v/>
       </c>
       <c r="F399" t="str">
-        <v>Admintrator</v>
+        <v/>
       </c>
       <c r="G399" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H399" t="str">
-        <v>VTS_H232VTS</v>
+        <v>An Dương Vương - 3</v>
       </c>
       <c r="I399" t="str">
-        <v>Trụ STK</v>
+        <v>Trụ bê tông đơn điện lực quản lý</v>
       </c>
       <c r="J399" t="str">
         <v/>
@@ -32274,16 +32274,16 @@
         <v>LED</v>
       </c>
       <c r="L399" t="str">
-        <v/>
+        <v>40</v>
       </c>
       <c r="M399" t="str">
         <v/>
       </c>
       <c r="N399" t="str">
-        <v>17:00:21 11/6/2026</v>
+        <v>16:09:49 6/7/2026</v>
       </c>
       <c r="O399" t="str">
-        <v/>
+        <v>H338.ADV_ADV_3_2</v>
       </c>
       <c r="P399" t="str">
         <v/>
@@ -32292,22 +32292,22 @@
         <v/>
       </c>
       <c r="R399" t="str">
-        <v/>
+        <v>Hẻm 338 An Dương Vương</v>
       </c>
       <c r="S399" t="str">
-        <v/>
+        <v>Phường 4</v>
       </c>
       <c r="T399" t="str">
-        <v>684316</v>
+        <v>683584</v>
       </c>
       <c r="U399" t="str">
-        <v>1192349</v>
+        <v>1189978</v>
       </c>
       <c r="V399" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W399" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X399" t="str">
         <v/>
@@ -32321,16 +32321,16 @@
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v/>
+        <v>41702_4</v>
       </c>
       <c r="B400" t="str">
-        <v/>
+        <v>H338.ADV_ADV_3_4</v>
       </c>
       <c r="C400" t="str">
-        <v/>
+        <v>10,7604271</v>
       </c>
       <c r="D400" t="str">
-        <v/>
+        <v>106,6788861</v>
       </c>
       <c r="E400" t="str">
         <v/>
@@ -32339,13 +32339,13 @@
         <v/>
       </c>
       <c r="G400" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H400" t="str">
-        <v>VTS_H232VTS</v>
+        <v>An Dương Vương - 3</v>
       </c>
       <c r="I400" t="str">
-        <v/>
+        <v>Trụ bê tông đơn điện lực quản lý</v>
       </c>
       <c r="J400" t="str">
         <v/>
@@ -32354,16 +32354,16 @@
         <v>LED</v>
       </c>
       <c r="L400" t="str">
-        <v/>
+        <v>40</v>
       </c>
       <c r="M400" t="str">
         <v/>
       </c>
       <c r="N400" t="str">
-        <v>16:36:28 15/6/2026</v>
+        <v>16:09:49 6/7/2026</v>
       </c>
       <c r="O400" t="str">
-        <v>VTS_H232VTS_15</v>
+        <v>H338.ADV_ADV_3_3</v>
       </c>
       <c r="P400" t="str">
         <v/>
@@ -32372,22 +32372,22 @@
         <v/>
       </c>
       <c r="R400" t="str">
-        <v/>
+        <v>Hẻm 338 An Dương Vương</v>
       </c>
       <c r="S400" t="str">
-        <v/>
+        <v>Phường 4</v>
       </c>
       <c r="T400" t="str">
-        <v>684302</v>
+        <v>683579</v>
       </c>
       <c r="U400" t="str">
-        <v>1192335</v>
+        <v>1189992</v>
       </c>
       <c r="V400" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W400" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X400" t="str">
         <v/>
@@ -32401,16 +32401,16 @@
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v/>
+        <v>41702_5</v>
       </c>
       <c r="B401" t="str">
-        <v/>
+        <v>H338.ADV_ADV_3_5</v>
       </c>
       <c r="C401" t="str">
-        <v/>
+        <v>10,7606929</v>
       </c>
       <c r="D401" t="str">
-        <v/>
+        <v>106,6788018</v>
       </c>
       <c r="E401" t="str">
         <v/>
@@ -32419,13 +32419,13 @@
         <v/>
       </c>
       <c r="G401" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H401" t="str">
-        <v>VTS_H232VTS</v>
+        <v>An Dương Vương - 3</v>
       </c>
       <c r="I401" t="str">
-        <v/>
+        <v>Trụ bê tông đơn điện lực quản lý</v>
       </c>
       <c r="J401" t="str">
         <v/>
@@ -32434,16 +32434,16 @@
         <v>LED</v>
       </c>
       <c r="L401" t="str">
-        <v/>
+        <v>40</v>
       </c>
       <c r="M401" t="str">
         <v/>
       </c>
       <c r="N401" t="str">
-        <v>16:36:30 15/6/2026</v>
+        <v>13:31:58 6/7/2026</v>
       </c>
       <c r="O401" t="str">
-        <v>VTS_H232VTS_16</v>
+        <v>H338.ADV_ADV_3_4</v>
       </c>
       <c r="P401" t="str">
         <v/>
@@ -32452,22 +32452,22 @@
         <v/>
       </c>
       <c r="R401" t="str">
-        <v/>
+        <v>Hẻm 338 An Dương Vương</v>
       </c>
       <c r="S401" t="str">
-        <v/>
+        <v>Phường 4</v>
       </c>
       <c r="T401" t="str">
-        <v>684282</v>
+        <v>683570</v>
       </c>
       <c r="U401" t="str">
-        <v>1192318</v>
+        <v>1190022</v>
       </c>
       <c r="V401" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W401" t="str">
-        <v/>
+        <v>noi</v>
       </c>
       <c r="X401" t="str">
         <v/>
@@ -32481,16 +32481,16 @@
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v/>
+        <v>T774.27148.093</v>
       </c>
       <c r="B402" t="str">
-        <v/>
+        <v xml:space="preserve">An Dương Vương - 3 </v>
       </c>
       <c r="C402" t="str">
-        <v/>
+        <v>10,7602173</v>
       </c>
       <c r="D402" t="str">
-        <v/>
+        <v>106,6807560</v>
       </c>
       <c r="E402" t="str">
         <v/>
@@ -32499,53 +32499,53 @@
         <v/>
       </c>
       <c r="G402" t="str">
+        <v>5</v>
+      </c>
+      <c r="H402" t="str">
+        <v xml:space="preserve">An Dương Vương - 3 </v>
+      </c>
+      <c r="I402" t="str">
+        <v/>
+      </c>
+      <c r="J402" t="str">
+        <v/>
+      </c>
+      <c r="K402" t="str">
+        <v/>
+      </c>
+      <c r="L402" t="str">
+        <v/>
+      </c>
+      <c r="M402" t="str">
+        <v/>
+      </c>
+      <c r="N402" t="str">
+        <v>13:19 23/06/2026</v>
+      </c>
+      <c r="O402" t="str">
+        <v/>
+      </c>
+      <c r="P402" t="str">
+        <v/>
+      </c>
+      <c r="Q402" t="str">
+        <v>PE03000082471</v>
+      </c>
+      <c r="R402" t="str">
+        <v>An Dương Vương</v>
+      </c>
+      <c r="S402" t="str">
+        <v>Phường 4</v>
+      </c>
+      <c r="T402" t="str">
+        <v>601600</v>
+      </c>
+      <c r="U402" t="str">
+        <v>1,19E+06</v>
+      </c>
+      <c r="V402" t="str">
         <v>1</v>
       </c>
-      <c r="H402" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I402" t="str">
-        <v/>
-      </c>
-      <c r="J402" t="str">
-        <v/>
-      </c>
-      <c r="K402" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L402" t="str">
-        <v/>
-      </c>
-      <c r="M402" t="str">
-        <v/>
-      </c>
-      <c r="N402" t="str">
-        <v>18:23:03 15/6/2026</v>
-      </c>
-      <c r="O402" t="str">
-        <v>VTS_H232VTS_17</v>
-      </c>
-      <c r="P402" t="str">
-        <v/>
-      </c>
-      <c r="Q402" t="str">
-        <v/>
-      </c>
-      <c r="R402" t="str">
-        <v/>
-      </c>
-      <c r="S402" t="str">
-        <v/>
-      </c>
-      <c r="T402" t="str">
-        <v>684262</v>
-      </c>
-      <c r="U402" t="str">
-        <v>1192297</v>
-      </c>
-      <c r="V402" t="str">
-        <v/>
-      </c>
       <c r="W402" t="str">
         <v/>
       </c>
@@ -32556,1852 +32556,12 @@
         <v/>
       </c>
       <c r="Z402" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="403">
-      <c r="A403" t="str">
-        <v/>
-      </c>
-      <c r="B403" t="str">
-        <v/>
-      </c>
-      <c r="C403" t="str">
-        <v/>
-      </c>
-      <c r="D403" t="str">
-        <v/>
-      </c>
-      <c r="E403" t="str">
-        <v/>
-      </c>
-      <c r="F403" t="str">
-        <v/>
-      </c>
-      <c r="G403" t="str">
-        <v>1</v>
-      </c>
-      <c r="H403" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I403" t="str">
-        <v/>
-      </c>
-      <c r="J403" t="str">
-        <v/>
-      </c>
-      <c r="K403" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L403" t="str">
-        <v/>
-      </c>
-      <c r="M403" t="str">
-        <v/>
-      </c>
-      <c r="N403" t="str">
-        <v>18:23:29 15/6/2026</v>
-      </c>
-      <c r="O403" t="str">
-        <v>VTS_H232VTS_18</v>
-      </c>
-      <c r="P403" t="str">
-        <v/>
-      </c>
-      <c r="Q403" t="str">
-        <v/>
-      </c>
-      <c r="R403" t="str">
-        <v/>
-      </c>
-      <c r="S403" t="str">
-        <v/>
-      </c>
-      <c r="T403" t="str">
-        <v>684237</v>
-      </c>
-      <c r="U403" t="str">
-        <v>1192270</v>
-      </c>
-      <c r="V403" t="str">
-        <v/>
-      </c>
-      <c r="W403" t="str">
-        <v/>
-      </c>
-      <c r="X403" t="str">
-        <v/>
-      </c>
-      <c r="Y403" t="str">
-        <v/>
-      </c>
-      <c r="Z403" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="404">
-      <c r="A404" t="str">
-        <v/>
-      </c>
-      <c r="B404" t="str">
-        <v/>
-      </c>
-      <c r="C404" t="str">
-        <v/>
-      </c>
-      <c r="D404" t="str">
-        <v/>
-      </c>
-      <c r="E404" t="str">
-        <v/>
-      </c>
-      <c r="F404" t="str">
-        <v/>
-      </c>
-      <c r="G404" t="str">
-        <v>1</v>
-      </c>
-      <c r="H404" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I404" t="str">
-        <v/>
-      </c>
-      <c r="J404" t="str">
-        <v/>
-      </c>
-      <c r="K404" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L404" t="str">
-        <v/>
-      </c>
-      <c r="M404" t="str">
-        <v/>
-      </c>
-      <c r="N404" t="str">
-        <v>11:29:09 11/6/2026</v>
-      </c>
-      <c r="O404" t="str">
-        <v>VTS_H232VTS_19</v>
-      </c>
-      <c r="P404" t="str">
-        <v/>
-      </c>
-      <c r="Q404" t="str">
-        <v/>
-      </c>
-      <c r="R404" t="str">
-        <v/>
-      </c>
-      <c r="S404" t="str">
-        <v/>
-      </c>
-      <c r="T404" t="str">
-        <v>684210</v>
-      </c>
-      <c r="U404" t="str">
-        <v>1192239</v>
-      </c>
-      <c r="V404" t="str">
-        <v/>
-      </c>
-      <c r="W404" t="str">
-        <v/>
-      </c>
-      <c r="X404" t="str">
-        <v/>
-      </c>
-      <c r="Y404" t="str">
-        <v/>
-      </c>
-      <c r="Z404" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="405">
-      <c r="A405" t="str">
-        <v/>
-      </c>
-      <c r="B405" t="str">
-        <v/>
-      </c>
-      <c r="C405" t="str">
-        <v/>
-      </c>
-      <c r="D405" t="str">
-        <v/>
-      </c>
-      <c r="E405" t="str">
-        <v/>
-      </c>
-      <c r="F405" t="str">
-        <v/>
-      </c>
-      <c r="G405" t="str">
-        <v>1</v>
-      </c>
-      <c r="H405" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I405" t="str">
-        <v/>
-      </c>
-      <c r="J405" t="str">
-        <v/>
-      </c>
-      <c r="K405" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L405" t="str">
-        <v/>
-      </c>
-      <c r="M405" t="str">
-        <v/>
-      </c>
-      <c r="N405" t="str">
-        <v>11:29:06 11/6/2026</v>
-      </c>
-      <c r="O405" t="str">
-        <v>VTS_H232VTS_20</v>
-      </c>
-      <c r="P405" t="str">
-        <v/>
-      </c>
-      <c r="Q405" t="str">
-        <v/>
-      </c>
-      <c r="R405" t="str">
-        <v/>
-      </c>
-      <c r="S405" t="str">
-        <v/>
-      </c>
-      <c r="T405" t="str">
-        <v>684195</v>
-      </c>
-      <c r="U405" t="str">
-        <v>1192223</v>
-      </c>
-      <c r="V405" t="str">
-        <v/>
-      </c>
-      <c r="W405" t="str">
-        <v/>
-      </c>
-      <c r="X405" t="str">
-        <v/>
-      </c>
-      <c r="Y405" t="str">
-        <v/>
-      </c>
-      <c r="Z405" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="406">
-      <c r="A406" t="str">
-        <v/>
-      </c>
-      <c r="B406" t="str">
-        <v/>
-      </c>
-      <c r="C406" t="str">
-        <v/>
-      </c>
-      <c r="D406" t="str">
-        <v/>
-      </c>
-      <c r="E406" t="str">
-        <v/>
-      </c>
-      <c r="F406" t="str">
-        <v/>
-      </c>
-      <c r="G406" t="str">
-        <v>1</v>
-      </c>
-      <c r="H406" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I406" t="str">
-        <v/>
-      </c>
-      <c r="J406" t="str">
-        <v/>
-      </c>
-      <c r="K406" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L406" t="str">
-        <v/>
-      </c>
-      <c r="M406" t="str">
-        <v/>
-      </c>
-      <c r="N406" t="str">
-        <v/>
-      </c>
-      <c r="O406" t="str">
-        <v>VTS_H232VTS_21</v>
-      </c>
-      <c r="P406" t="str">
-        <v/>
-      </c>
-      <c r="Q406" t="str">
-        <v/>
-      </c>
-      <c r="R406" t="str">
-        <v/>
-      </c>
-      <c r="S406" t="str">
-        <v/>
-      </c>
-      <c r="T406" t="str">
-        <v>684176</v>
-      </c>
-      <c r="U406" t="str">
-        <v>1192205</v>
-      </c>
-      <c r="V406" t="str">
-        <v/>
-      </c>
-      <c r="W406" t="str">
-        <v/>
-      </c>
-      <c r="X406" t="str">
-        <v/>
-      </c>
-      <c r="Y406" t="str">
-        <v/>
-      </c>
-      <c r="Z406" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="407">
-      <c r="A407" t="str">
-        <v/>
-      </c>
-      <c r="B407" t="str">
-        <v/>
-      </c>
-      <c r="C407" t="str">
-        <v/>
-      </c>
-      <c r="D407" t="str">
-        <v/>
-      </c>
-      <c r="E407" t="str">
-        <v/>
-      </c>
-      <c r="F407" t="str">
-        <v/>
-      </c>
-      <c r="G407" t="str">
-        <v>1</v>
-      </c>
-      <c r="H407" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I407" t="str">
-        <v/>
-      </c>
-      <c r="J407" t="str">
-        <v/>
-      </c>
-      <c r="K407" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L407" t="str">
-        <v/>
-      </c>
-      <c r="M407" t="str">
-        <v/>
-      </c>
-      <c r="N407" t="str">
-        <v>16:02:09 10/6/2026</v>
-      </c>
-      <c r="O407" t="str">
-        <v>VTS_H232VTS_22</v>
-      </c>
-      <c r="P407" t="str">
-        <v/>
-      </c>
-      <c r="Q407" t="str">
-        <v/>
-      </c>
-      <c r="R407" t="str">
-        <v/>
-      </c>
-      <c r="S407" t="str">
-        <v/>
-      </c>
-      <c r="T407" t="str">
-        <v>684154</v>
-      </c>
-      <c r="U407" t="str">
-        <v>1192182</v>
-      </c>
-      <c r="V407" t="str">
-        <v/>
-      </c>
-      <c r="W407" t="str">
-        <v/>
-      </c>
-      <c r="X407" t="str">
-        <v/>
-      </c>
-      <c r="Y407" t="str">
-        <v/>
-      </c>
-      <c r="Z407" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="408">
-      <c r="A408" t="str">
-        <v/>
-      </c>
-      <c r="B408" t="str">
-        <v/>
-      </c>
-      <c r="C408" t="str">
-        <v/>
-      </c>
-      <c r="D408" t="str">
-        <v/>
-      </c>
-      <c r="E408" t="str">
-        <v/>
-      </c>
-      <c r="F408" t="str">
-        <v/>
-      </c>
-      <c r="G408" t="str">
-        <v>1</v>
-      </c>
-      <c r="H408" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I408" t="str">
-        <v/>
-      </c>
-      <c r="J408" t="str">
-        <v/>
-      </c>
-      <c r="K408" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L408" t="str">
-        <v/>
-      </c>
-      <c r="M408" t="str">
-        <v/>
-      </c>
-      <c r="N408" t="str">
-        <v/>
-      </c>
-      <c r="O408" t="str">
-        <v>VTS_H232VTS_23</v>
-      </c>
-      <c r="P408" t="str">
-        <v/>
-      </c>
-      <c r="Q408" t="str">
-        <v/>
-      </c>
-      <c r="R408" t="str">
-        <v/>
-      </c>
-      <c r="S408" t="str">
-        <v/>
-      </c>
-      <c r="T408" t="str">
-        <v>684130</v>
-      </c>
-      <c r="U408" t="str">
-        <v>1192158</v>
-      </c>
-      <c r="V408" t="str">
-        <v/>
-      </c>
-      <c r="W408" t="str">
-        <v/>
-      </c>
-      <c r="X408" t="str">
-        <v/>
-      </c>
-      <c r="Y408" t="str">
-        <v/>
-      </c>
-      <c r="Z408" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="409">
-      <c r="A409" t="str">
-        <v/>
-      </c>
-      <c r="B409" t="str">
-        <v/>
-      </c>
-      <c r="C409" t="str">
-        <v/>
-      </c>
-      <c r="D409" t="str">
-        <v/>
-      </c>
-      <c r="E409" t="str">
-        <v/>
-      </c>
-      <c r="F409" t="str">
-        <v/>
-      </c>
-      <c r="G409" t="str">
-        <v>1</v>
-      </c>
-      <c r="H409" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I409" t="str">
-        <v/>
-      </c>
-      <c r="J409" t="str">
-        <v/>
-      </c>
-      <c r="K409" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L409" t="str">
-        <v/>
-      </c>
-      <c r="M409" t="str">
-        <v/>
-      </c>
-      <c r="N409" t="str">
-        <v>11:29:01 11/6/2026</v>
-      </c>
-      <c r="O409" t="str">
-        <v>VTS_H232VTS_24</v>
-      </c>
-      <c r="P409" t="str">
-        <v/>
-      </c>
-      <c r="Q409" t="str">
-        <v/>
-      </c>
-      <c r="R409" t="str">
-        <v/>
-      </c>
-      <c r="S409" t="str">
-        <v/>
-      </c>
-      <c r="T409" t="str">
-        <v>684111</v>
-      </c>
-      <c r="U409" t="str">
-        <v>1192139</v>
-      </c>
-      <c r="V409" t="str">
-        <v/>
-      </c>
-      <c r="W409" t="str">
-        <v/>
-      </c>
-      <c r="X409" t="str">
-        <v/>
-      </c>
-      <c r="Y409" t="str">
-        <v/>
-      </c>
-      <c r="Z409" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="410">
-      <c r="A410" t="str">
-        <v/>
-      </c>
-      <c r="B410" t="str">
-        <v/>
-      </c>
-      <c r="C410" t="str">
-        <v/>
-      </c>
-      <c r="D410" t="str">
-        <v/>
-      </c>
-      <c r="E410" t="str">
-        <v/>
-      </c>
-      <c r="F410" t="str">
-        <v/>
-      </c>
-      <c r="G410" t="str">
-        <v>1</v>
-      </c>
-      <c r="H410" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I410" t="str">
-        <v/>
-      </c>
-      <c r="J410" t="str">
-        <v/>
-      </c>
-      <c r="K410" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L410" t="str">
-        <v/>
-      </c>
-      <c r="M410" t="str">
-        <v/>
-      </c>
-      <c r="N410" t="str">
-        <v>16:01:17 10/6/2026</v>
-      </c>
-      <c r="O410" t="str">
-        <v>VTS_H232VTS_25</v>
-      </c>
-      <c r="P410" t="str">
-        <v/>
-      </c>
-      <c r="Q410" t="str">
-        <v/>
-      </c>
-      <c r="R410" t="str">
-        <v/>
-      </c>
-      <c r="S410" t="str">
-        <v/>
-      </c>
-      <c r="T410" t="str">
-        <v>684094</v>
-      </c>
-      <c r="U410" t="str">
-        <v>1192120</v>
-      </c>
-      <c r="V410" t="str">
-        <v/>
-      </c>
-      <c r="W410" t="str">
-        <v/>
-      </c>
-      <c r="X410" t="str">
-        <v/>
-      </c>
-      <c r="Y410" t="str">
-        <v/>
-      </c>
-      <c r="Z410" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="411">
-      <c r="A411" t="str">
-        <v/>
-      </c>
-      <c r="B411" t="str">
-        <v/>
-      </c>
-      <c r="C411" t="str">
-        <v/>
-      </c>
-      <c r="D411" t="str">
-        <v/>
-      </c>
-      <c r="E411" t="str">
-        <v/>
-      </c>
-      <c r="F411" t="str">
-        <v/>
-      </c>
-      <c r="G411" t="str">
-        <v>1</v>
-      </c>
-      <c r="H411" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I411" t="str">
-        <v/>
-      </c>
-      <c r="J411" t="str">
-        <v/>
-      </c>
-      <c r="K411" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L411" t="str">
-        <v/>
-      </c>
-      <c r="M411" t="str">
-        <v/>
-      </c>
-      <c r="N411" t="str">
-        <v>16:01:12 10/6/2026</v>
-      </c>
-      <c r="O411" t="str">
-        <v>VTS_H232VTS_26</v>
-      </c>
-      <c r="P411" t="str">
-        <v/>
-      </c>
-      <c r="Q411" t="str">
-        <v/>
-      </c>
-      <c r="R411" t="str">
-        <v/>
-      </c>
-      <c r="S411" t="str">
-        <v/>
-      </c>
-      <c r="T411" t="str">
-        <v>684067</v>
-      </c>
-      <c r="U411" t="str">
-        <v>1192094</v>
-      </c>
-      <c r="V411" t="str">
-        <v/>
-      </c>
-      <c r="W411" t="str">
-        <v/>
-      </c>
-      <c r="X411" t="str">
-        <v/>
-      </c>
-      <c r="Y411" t="str">
-        <v/>
-      </c>
-      <c r="Z411" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="412">
-      <c r="A412" t="str">
-        <v/>
-      </c>
-      <c r="B412" t="str">
-        <v/>
-      </c>
-      <c r="C412" t="str">
-        <v/>
-      </c>
-      <c r="D412" t="str">
-        <v/>
-      </c>
-      <c r="E412" t="str">
-        <v/>
-      </c>
-      <c r="F412" t="str">
-        <v/>
-      </c>
-      <c r="G412" t="str">
-        <v>1</v>
-      </c>
-      <c r="H412" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I412" t="str">
-        <v/>
-      </c>
-      <c r="J412" t="str">
-        <v/>
-      </c>
-      <c r="K412" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L412" t="str">
-        <v/>
-      </c>
-      <c r="M412" t="str">
-        <v/>
-      </c>
-      <c r="N412" t="str">
-        <v>15:58:28 12/6/2026</v>
-      </c>
-      <c r="O412" t="str">
-        <v>VTS_H232VTS_27</v>
-      </c>
-      <c r="P412" t="str">
-        <v/>
-      </c>
-      <c r="Q412" t="str">
-        <v/>
-      </c>
-      <c r="R412" t="str">
-        <v/>
-      </c>
-      <c r="S412" t="str">
-        <v/>
-      </c>
-      <c r="T412" t="str">
-        <v>684046</v>
-      </c>
-      <c r="U412" t="str">
-        <v>1192073</v>
-      </c>
-      <c r="V412" t="str">
-        <v/>
-      </c>
-      <c r="W412" t="str">
-        <v/>
-      </c>
-      <c r="X412" t="str">
-        <v/>
-      </c>
-      <c r="Y412" t="str">
-        <v/>
-      </c>
-      <c r="Z412" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="413">
-      <c r="A413" t="str">
-        <v/>
-      </c>
-      <c r="B413" t="str">
-        <v/>
-      </c>
-      <c r="C413" t="str">
-        <v/>
-      </c>
-      <c r="D413" t="str">
-        <v/>
-      </c>
-      <c r="E413" t="str">
-        <v/>
-      </c>
-      <c r="F413" t="str">
-        <v/>
-      </c>
-      <c r="G413" t="str">
-        <v>1</v>
-      </c>
-      <c r="H413" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I413" t="str">
-        <v/>
-      </c>
-      <c r="J413" t="str">
-        <v/>
-      </c>
-      <c r="K413" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L413" t="str">
-        <v/>
-      </c>
-      <c r="M413" t="str">
-        <v/>
-      </c>
-      <c r="N413" t="str">
-        <v>13:18:19 12/6/2026</v>
-      </c>
-      <c r="O413" t="str">
-        <v>VTS_H232VTS_28</v>
-      </c>
-      <c r="P413" t="str">
-        <v/>
-      </c>
-      <c r="Q413" t="str">
-        <v/>
-      </c>
-      <c r="R413" t="str">
-        <v/>
-      </c>
-      <c r="S413" t="str">
-        <v/>
-      </c>
-      <c r="T413" t="str">
-        <v>684021</v>
-      </c>
-      <c r="U413" t="str">
-        <v>1192048</v>
-      </c>
-      <c r="V413" t="str">
-        <v/>
-      </c>
-      <c r="W413" t="str">
-        <v/>
-      </c>
-      <c r="X413" t="str">
-        <v/>
-      </c>
-      <c r="Y413" t="str">
-        <v/>
-      </c>
-      <c r="Z413" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" t="str">
-        <v/>
-      </c>
-      <c r="B414" t="str">
-        <v/>
-      </c>
-      <c r="C414" t="str">
-        <v/>
-      </c>
-      <c r="D414" t="str">
-        <v/>
-      </c>
-      <c r="E414" t="str">
-        <v/>
-      </c>
-      <c r="F414" t="str">
-        <v/>
-      </c>
-      <c r="G414" t="str">
-        <v>1</v>
-      </c>
-      <c r="H414" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I414" t="str">
-        <v/>
-      </c>
-      <c r="J414" t="str">
-        <v/>
-      </c>
-      <c r="K414" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L414" t="str">
-        <v/>
-      </c>
-      <c r="M414" t="str">
-        <v/>
-      </c>
-      <c r="N414" t="str">
-        <v>13:18:21 12/6/2026</v>
-      </c>
-      <c r="O414" t="str">
-        <v>VTS_H232VTS_29</v>
-      </c>
-      <c r="P414" t="str">
-        <v/>
-      </c>
-      <c r="Q414" t="str">
-        <v/>
-      </c>
-      <c r="R414" t="str">
-        <v/>
-      </c>
-      <c r="S414" t="str">
-        <v/>
-      </c>
-      <c r="T414" t="str">
-        <v>683993</v>
-      </c>
-      <c r="U414" t="str">
-        <v>1192018</v>
-      </c>
-      <c r="V414" t="str">
-        <v/>
-      </c>
-      <c r="W414" t="str">
-        <v/>
-      </c>
-      <c r="X414" t="str">
-        <v/>
-      </c>
-      <c r="Y414" t="str">
-        <v/>
-      </c>
-      <c r="Z414" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="415">
-      <c r="A415" t="str">
-        <v/>
-      </c>
-      <c r="B415" t="str">
-        <v/>
-      </c>
-      <c r="C415" t="str">
-        <v/>
-      </c>
-      <c r="D415" t="str">
-        <v/>
-      </c>
-      <c r="E415" t="str">
-        <v/>
-      </c>
-      <c r="F415" t="str">
-        <v/>
-      </c>
-      <c r="G415" t="str">
-        <v>1</v>
-      </c>
-      <c r="H415" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I415" t="str">
-        <v/>
-      </c>
-      <c r="J415" t="str">
-        <v/>
-      </c>
-      <c r="K415" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L415" t="str">
-        <v/>
-      </c>
-      <c r="M415" t="str">
-        <v/>
-      </c>
-      <c r="N415" t="str">
-        <v>13:20:36 12/6/2026</v>
-      </c>
-      <c r="O415" t="str">
-        <v>VTS_H232VTS_30</v>
-      </c>
-      <c r="P415" t="str">
-        <v/>
-      </c>
-      <c r="Q415" t="str">
-        <v/>
-      </c>
-      <c r="R415" t="str">
-        <v/>
-      </c>
-      <c r="S415" t="str">
-        <v/>
-      </c>
-      <c r="T415" t="str">
-        <v>683974</v>
-      </c>
-      <c r="U415" t="str">
-        <v>1191996</v>
-      </c>
-      <c r="V415" t="str">
-        <v/>
-      </c>
-      <c r="W415" t="str">
-        <v/>
-      </c>
-      <c r="X415" t="str">
-        <v/>
-      </c>
-      <c r="Y415" t="str">
-        <v/>
-      </c>
-      <c r="Z415" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="416">
-      <c r="A416" t="str">
-        <v/>
-      </c>
-      <c r="B416" t="str">
-        <v/>
-      </c>
-      <c r="C416" t="str">
-        <v/>
-      </c>
-      <c r="D416" t="str">
-        <v/>
-      </c>
-      <c r="E416" t="str">
-        <v/>
-      </c>
-      <c r="F416" t="str">
-        <v/>
-      </c>
-      <c r="G416" t="str">
-        <v>1</v>
-      </c>
-      <c r="H416" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I416" t="str">
-        <v/>
-      </c>
-      <c r="J416" t="str">
-        <v/>
-      </c>
-      <c r="K416" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L416" t="str">
-        <v/>
-      </c>
-      <c r="M416" t="str">
-        <v/>
-      </c>
-      <c r="N416" t="str">
-        <v>13:20:39 12/6/2026</v>
-      </c>
-      <c r="O416" t="str">
-        <v>VTS_H232VTS_31</v>
-      </c>
-      <c r="P416" t="str">
-        <v/>
-      </c>
-      <c r="Q416" t="str">
-        <v/>
-      </c>
-      <c r="R416" t="str">
-        <v/>
-      </c>
-      <c r="S416" t="str">
-        <v/>
-      </c>
-      <c r="T416" t="str">
-        <v>683958</v>
-      </c>
-      <c r="U416" t="str">
-        <v>1191980</v>
-      </c>
-      <c r="V416" t="str">
-        <v/>
-      </c>
-      <c r="W416" t="str">
-        <v/>
-      </c>
-      <c r="X416" t="str">
-        <v/>
-      </c>
-      <c r="Y416" t="str">
-        <v/>
-      </c>
-      <c r="Z416" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" t="str">
-        <v/>
-      </c>
-      <c r="B417" t="str">
-        <v/>
-      </c>
-      <c r="C417" t="str">
-        <v/>
-      </c>
-      <c r="D417" t="str">
-        <v/>
-      </c>
-      <c r="E417" t="str">
-        <v/>
-      </c>
-      <c r="F417" t="str">
-        <v/>
-      </c>
-      <c r="G417" t="str">
-        <v>1</v>
-      </c>
-      <c r="H417" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I417" t="str">
-        <v/>
-      </c>
-      <c r="J417" t="str">
-        <v/>
-      </c>
-      <c r="K417" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L417" t="str">
-        <v/>
-      </c>
-      <c r="M417" t="str">
-        <v/>
-      </c>
-      <c r="N417" t="str">
-        <v>15:58:02 12/6/2026</v>
-      </c>
-      <c r="O417" t="str">
-        <v>VTS_H232VTS_32</v>
-      </c>
-      <c r="P417" t="str">
-        <v/>
-      </c>
-      <c r="Q417" t="str">
-        <v/>
-      </c>
-      <c r="R417" t="str">
-        <v/>
-      </c>
-      <c r="S417" t="str">
-        <v/>
-      </c>
-      <c r="T417" t="str">
-        <v>683943</v>
-      </c>
-      <c r="U417" t="str">
-        <v>1191964</v>
-      </c>
-      <c r="V417" t="str">
-        <v/>
-      </c>
-      <c r="W417" t="str">
-        <v/>
-      </c>
-      <c r="X417" t="str">
-        <v/>
-      </c>
-      <c r="Y417" t="str">
-        <v/>
-      </c>
-      <c r="Z417" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="418">
-      <c r="A418" t="str">
-        <v/>
-      </c>
-      <c r="B418" t="str">
-        <v/>
-      </c>
-      <c r="C418" t="str">
-        <v/>
-      </c>
-      <c r="D418" t="str">
-        <v/>
-      </c>
-      <c r="E418" t="str">
-        <v/>
-      </c>
-      <c r="F418" t="str">
-        <v/>
-      </c>
-      <c r="G418" t="str">
-        <v>1</v>
-      </c>
-      <c r="H418" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I418" t="str">
-        <v/>
-      </c>
-      <c r="J418" t="str">
-        <v/>
-      </c>
-      <c r="K418" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L418" t="str">
-        <v/>
-      </c>
-      <c r="M418" t="str">
-        <v/>
-      </c>
-      <c r="N418" t="str">
-        <v>15:57:52 12/6/2026</v>
-      </c>
-      <c r="O418" t="str">
-        <v>VTS_H232VTS_33</v>
-      </c>
-      <c r="P418" t="str">
-        <v/>
-      </c>
-      <c r="Q418" t="str">
-        <v/>
-      </c>
-      <c r="R418" t="str">
-        <v/>
-      </c>
-      <c r="S418" t="str">
-        <v/>
-      </c>
-      <c r="T418" t="str">
-        <v>683918</v>
-      </c>
-      <c r="U418" t="str">
-        <v>1191942</v>
-      </c>
-      <c r="V418" t="str">
-        <v/>
-      </c>
-      <c r="W418" t="str">
-        <v/>
-      </c>
-      <c r="X418" t="str">
-        <v/>
-      </c>
-      <c r="Y418" t="str">
-        <v/>
-      </c>
-      <c r="Z418" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="419">
-      <c r="A419" t="str">
-        <v/>
-      </c>
-      <c r="B419" t="str">
-        <v/>
-      </c>
-      <c r="C419" t="str">
-        <v/>
-      </c>
-      <c r="D419" t="str">
-        <v/>
-      </c>
-      <c r="E419" t="str">
-        <v/>
-      </c>
-      <c r="F419" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G419" t="str">
-        <v>6</v>
-      </c>
-      <c r="H419" t="str">
-        <v>VTS_H232VTS</v>
-      </c>
-      <c r="I419" t="str">
-        <v>Tủ chiếu sáng ngầm</v>
-      </c>
-      <c r="J419" t="str">
-        <v/>
-      </c>
-      <c r="K419" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L419" t="str">
-        <v/>
-      </c>
-      <c r="M419" t="str">
-        <v/>
-      </c>
-      <c r="N419" t="str">
-        <v>16:36:37 15/6/2026</v>
-      </c>
-      <c r="O419" t="str">
-        <v>VTS_H232VTS_14</v>
-      </c>
-      <c r="P419" t="str">
-        <v>12</v>
-      </c>
-      <c r="Q419" t="str">
-        <v/>
-      </c>
-      <c r="R419" t="str">
-        <v>Đường Võ Thị Sáu</v>
-      </c>
-      <c r="S419" t="str">
-        <v>Phường Xuân Hòa</v>
-      </c>
-      <c r="T419" t="str">
-        <v>684326</v>
-      </c>
-      <c r="U419" t="str">
-        <v>1192362</v>
-      </c>
-      <c r="V419" t="str">
-        <v/>
-      </c>
-      <c r="W419" t="str">
-        <v/>
-      </c>
-      <c r="X419" t="str">
-        <v/>
-      </c>
-      <c r="Y419" t="str">
-        <v/>
-      </c>
-      <c r="Z419" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="420">
-      <c r="A420" t="str">
-        <v/>
-      </c>
-      <c r="B420" t="str">
-        <v/>
-      </c>
-      <c r="C420" t="str">
-        <v/>
-      </c>
-      <c r="D420" t="str">
-        <v/>
-      </c>
-      <c r="E420" t="str">
-        <v/>
-      </c>
-      <c r="F420" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G420" t="str">
-        <v>1</v>
-      </c>
-      <c r="H420" t="str">
-        <v>Tân Khai</v>
-      </c>
-      <c r="I420" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J420" t="str">
-        <v/>
-      </c>
-      <c r="K420" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L420" t="str">
-        <v>90</v>
-      </c>
-      <c r="M420" t="str">
-        <v/>
-      </c>
-      <c r="N420" t="str">
-        <v>08:04:34 14/6/2026</v>
-      </c>
-      <c r="O420" t="str">
-        <v>Tk 1</v>
-      </c>
-      <c r="P420" t="str">
-        <v>0</v>
-      </c>
-      <c r="Q420" t="str">
-        <v/>
-      </c>
-      <c r="R420" t="str">
-        <v/>
-      </c>
-      <c r="S420" t="str">
-        <v>Phường Tân Khai</v>
-      </c>
-      <c r="T420" t="str">
-        <v>675958</v>
-      </c>
-      <c r="U420" t="str">
-        <v>1279166</v>
-      </c>
-      <c r="V420" t="str">
-        <v>1</v>
-      </c>
-      <c r="W420" t="str">
-        <v/>
-      </c>
-      <c r="X420" t="str">
-        <v/>
-      </c>
-      <c r="Y420" t="str">
-        <v/>
-      </c>
-      <c r="Z420" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" t="str">
-        <v/>
-      </c>
-      <c r="B421" t="str">
-        <v/>
-      </c>
-      <c r="C421" t="str">
-        <v/>
-      </c>
-      <c r="D421" t="str">
-        <v/>
-      </c>
-      <c r="E421" t="str">
-        <v/>
-      </c>
-      <c r="F421" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G421" t="str">
-        <v>1</v>
-      </c>
-      <c r="H421" t="str">
-        <v>Tân Khai</v>
-      </c>
-      <c r="I421" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J421" t="str">
-        <v/>
-      </c>
-      <c r="K421" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L421" t="str">
-        <v>90</v>
-      </c>
-      <c r="M421" t="str">
-        <v/>
-      </c>
-      <c r="N421" t="str">
-        <v>11:28:07 15/6/2026</v>
-      </c>
-      <c r="O421" t="str">
-        <v>Tk 2</v>
-      </c>
-      <c r="P421" t="str">
-        <v>4</v>
-      </c>
-      <c r="Q421" t="str">
-        <v/>
-      </c>
-      <c r="R421" t="str">
-        <v/>
-      </c>
-      <c r="S421" t="str">
-        <v>Phường Tân Khai</v>
-      </c>
-      <c r="T421" t="str">
-        <v>675969</v>
-      </c>
-      <c r="U421" t="str">
-        <v>1279297</v>
-      </c>
-      <c r="V421" t="str">
-        <v>1</v>
-      </c>
-      <c r="W421" t="str">
-        <v/>
-      </c>
-      <c r="X421" t="str">
-        <v/>
-      </c>
-      <c r="Y421" t="str">
-        <v/>
-      </c>
-      <c r="Z421" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="422">
-      <c r="A422" t="str">
-        <v/>
-      </c>
-      <c r="B422" t="str">
-        <v/>
-      </c>
-      <c r="C422" t="str">
-        <v/>
-      </c>
-      <c r="D422" t="str">
-        <v/>
-      </c>
-      <c r="E422" t="str">
-        <v/>
-      </c>
-      <c r="F422" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G422" t="str">
-        <v>1</v>
-      </c>
-      <c r="H422" t="str">
-        <v>Tân Khai</v>
-      </c>
-      <c r="I422" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J422" t="str">
-        <v/>
-      </c>
-      <c r="K422" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L422" t="str">
-        <v>90</v>
-      </c>
-      <c r="M422" t="str">
-        <v/>
-      </c>
-      <c r="N422" t="str">
-        <v>11:28:35 15/6/2026</v>
-      </c>
-      <c r="O422" t="str">
-        <v>Tk 2</v>
-      </c>
-      <c r="P422" t="str">
-        <v>5</v>
-      </c>
-      <c r="Q422" t="str">
-        <v/>
-      </c>
-      <c r="R422" t="str">
-        <v/>
-      </c>
-      <c r="S422" t="str">
-        <v>Phường Tân Khai</v>
-      </c>
-      <c r="T422" t="str">
-        <v>675969</v>
-      </c>
-      <c r="U422" t="str">
-        <v>1279296</v>
-      </c>
-      <c r="V422" t="str">
-        <v>1</v>
-      </c>
-      <c r="W422" t="str">
-        <v/>
-      </c>
-      <c r="X422" t="str">
-        <v/>
-      </c>
-      <c r="Y422" t="str">
-        <v/>
-      </c>
-      <c r="Z422" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="423">
-      <c r="A423" t="str">
-        <v/>
-      </c>
-      <c r="B423" t="str">
-        <v/>
-      </c>
-      <c r="C423" t="str">
-        <v/>
-      </c>
-      <c r="D423" t="str">
-        <v/>
-      </c>
-      <c r="E423" t="str">
-        <v/>
-      </c>
-      <c r="F423" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G423" t="str">
-        <v>1</v>
-      </c>
-      <c r="H423" t="str">
-        <v>Tân Khai</v>
-      </c>
-      <c r="I423" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J423" t="str">
-        <v/>
-      </c>
-      <c r="K423" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L423" t="str">
-        <v>90</v>
-      </c>
-      <c r="M423" t="str">
-        <v/>
-      </c>
-      <c r="N423" t="str">
-        <v>11:27:21 15/6/2026</v>
-      </c>
-      <c r="O423" t="str">
-        <v>Tk 3</v>
-      </c>
-      <c r="P423" t="str">
-        <v>50</v>
-      </c>
-      <c r="Q423" t="str">
-        <v/>
-      </c>
-      <c r="R423" t="str">
-        <v/>
-      </c>
-      <c r="S423" t="str">
-        <v>Phường Tân Khai</v>
-      </c>
-      <c r="T423" t="str">
-        <v>675946</v>
-      </c>
-      <c r="U423" t="str">
-        <v>1279262</v>
-      </c>
-      <c r="V423" t="str">
-        <v>1</v>
-      </c>
-      <c r="W423" t="str">
-        <v/>
-      </c>
-      <c r="X423" t="str">
-        <v/>
-      </c>
-      <c r="Y423" t="str">
-        <v/>
-      </c>
-      <c r="Z423" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="424">
-      <c r="A424" t="str">
-        <v/>
-      </c>
-      <c r="B424" t="str">
-        <v/>
-      </c>
-      <c r="C424" t="str">
-        <v/>
-      </c>
-      <c r="D424" t="str">
-        <v/>
-      </c>
-      <c r="E424" t="str">
-        <v/>
-      </c>
-      <c r="F424" t="str">
-        <v>Admintrator</v>
-      </c>
-      <c r="G424" t="str">
-        <v>1</v>
-      </c>
-      <c r="H424" t="str">
-        <v/>
-      </c>
-      <c r="I424" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J424" t="str">
-        <v/>
-      </c>
-      <c r="K424" t="str">
-        <v/>
-      </c>
-      <c r="L424" t="str">
-        <v/>
-      </c>
-      <c r="M424" t="str">
-        <v/>
-      </c>
-      <c r="N424" t="str">
-        <v>15:17:55 18/6/2026</v>
-      </c>
-      <c r="O424" t="str">
-        <v/>
-      </c>
-      <c r="P424" t="str">
-        <v/>
-      </c>
-      <c r="Q424" t="str">
-        <v/>
-      </c>
-      <c r="R424" t="str">
-        <v>Lê Quang Đạo</v>
-      </c>
-      <c r="S424" t="str">
-        <v/>
-      </c>
-      <c r="T424" t="str">
-        <v>673401</v>
-      </c>
-      <c r="U424" t="str">
-        <v>1203667</v>
-      </c>
-      <c r="V424" t="str">
-        <v/>
-      </c>
-      <c r="W424" t="str">
-        <v>noi</v>
-      </c>
-      <c r="X424" t="str">
-        <v/>
-      </c>
-      <c r="Y424" t="str">
-        <v/>
-      </c>
-      <c r="Z424" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="425">
-      <c r="A425" t="str">
-        <v/>
-      </c>
-      <c r="B425" t="str">
-        <v/>
-      </c>
-      <c r="C425" t="str">
-        <v/>
-      </c>
-      <c r="D425" t="str">
-        <v/>
-      </c>
-      <c r="E425" t="str">
-        <v/>
-      </c>
-      <c r="F425" t="str">
-        <v>P.KTHTCG</v>
-      </c>
-      <c r="G425" t="str">
-        <v>1</v>
-      </c>
-      <c r="H425" t="str">
-        <v>Tủ D41</v>
-      </c>
-      <c r="I425" t="str">
-        <v>Trụ STK</v>
-      </c>
-      <c r="J425" t="str">
-        <v/>
-      </c>
-      <c r="K425" t="str">
-        <v>LED</v>
-      </c>
-      <c r="L425" t="str">
-        <v>150</v>
-      </c>
-      <c r="M425" t="str">
-        <v/>
-      </c>
-      <c r="N425" t="str">
-        <v>15:49:50 21/6/2026</v>
-      </c>
-      <c r="O425" t="str">
-        <v/>
-      </c>
-      <c r="P425" t="str">
-        <v/>
-      </c>
-      <c r="Q425" t="str">
-        <v/>
-      </c>
-      <c r="R425" t="str">
-        <v>ĐT.835</v>
-      </c>
-      <c r="S425" t="str">
-        <v>Cần Giuộc</v>
-      </c>
-      <c r="T425" t="str">
-        <v>657144</v>
-      </c>
-      <c r="U425" t="str">
-        <v>1164284</v>
-      </c>
-      <c r="V425" t="str">
-        <v>5</v>
-      </c>
-      <c r="W425" t="str">
-        <v>noi</v>
-      </c>
-      <c r="X425" t="str">
-        <v/>
-      </c>
-      <c r="Y425" t="str">
-        <v/>
-      </c>
-      <c r="Z425" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z425"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z402"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>